<commit_message>
added branch for testing
</commit_message>
<xml_diff>
--- a/src/results/GWP/optimized_results_GWP.xlsx
+++ b/src/results/GWP/optimized_results_GWP.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D121"/>
+  <dimension ref="A1:E121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,6 +435,11 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Unit</t>
         </is>
       </c>
@@ -448,6 +453,7 @@
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr"/>
@@ -459,7 +465,10 @@
       <c r="C3" t="n">
         <v>15</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>m</t>
         </is>
@@ -469,13 +478,16 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Chrod length</t>
+          <t>Chord length</t>
         </is>
       </c>
       <c r="C4" t="n">
         <v>1.718</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="n">
+        <v>1.718</v>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>m</t>
         </is>
@@ -491,7 +503,10 @@
       <c r="C5" t="n">
         <v>1.569</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="n">
+        <v>1.569</v>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>m</t>
         </is>
@@ -507,7 +522,10 @@
       <c r="C6" t="n">
         <v>1.567</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" t="n">
+        <v>1.567</v>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>m</t>
         </is>
@@ -517,13 +535,16 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>battery energy density</t>
+          <t>Battery energy density</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>400</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" t="n">
+        <v>400</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>Wh/kg</t>
         </is>
@@ -539,7 +560,10 @@
       <c r="C8" t="n">
         <v>1</v>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>1/h</t>
         </is>
@@ -554,6 +578,7 @@
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr"/>
@@ -565,7 +590,10 @@
       <c r="C10" t="n">
         <v>8.731999999999999</v>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" t="n">
+        <v>8.731999999999999</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -581,7 +609,10 @@
       <c r="C11" t="n">
         <v>0.522</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" t="n">
+        <v>0.522</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -597,7 +628,10 @@
       <c r="C12" t="n">
         <v>0.052</v>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -613,7 +647,10 @@
       <c r="C13" t="n">
         <v>10.015</v>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" t="n">
+        <v>10.015</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -629,7 +666,10 @@
       <c r="C14" t="n">
         <v>1517.469</v>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" t="n">
+        <v>1517.469</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -645,7 +685,10 @@
       <c r="C15" t="n">
         <v>0.919</v>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" t="n">
+        <v>0.919</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -661,7 +704,10 @@
       <c r="C16" t="n">
         <v>0.078</v>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" t="n">
+        <v>0.078</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -677,7 +723,10 @@
       <c r="C17" t="n">
         <v>11.754</v>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" t="n">
+        <v>11.754</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -693,7 +742,10 @@
       <c r="C18" t="n">
         <v>1286.997</v>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" t="n">
+        <v>1286.997</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -708,6 +760,7 @@
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
@@ -719,7 +772,10 @@
       <c r="C20" t="n">
         <v>42.955</v>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" t="n">
+        <v>42.955</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
@@ -735,7 +791,10 @@
       <c r="C21" t="n">
         <v>32.29</v>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" t="n">
+        <v>32.29</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
@@ -751,7 +810,10 @@
       <c r="C22" t="n">
         <v>31.976</v>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" t="n">
+        <v>31.976</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
@@ -767,7 +829,10 @@
       <c r="C23" t="n">
         <v>4.494</v>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" t="n">
+        <v>4.494</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
@@ -782,6 +847,7 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
@@ -793,7 +859,10 @@
       <c r="C25" t="n">
         <v>3413.082</v>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" t="n">
+        <v>3413.082</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -809,7 +878,10 @@
       <c r="C26" t="n">
         <v>3413.082</v>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" t="n">
+        <v>3413.082</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -825,7 +897,10 @@
       <c r="C27" t="n">
         <v>165712.862</v>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" t="n">
+        <v>165712.862</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>W</t>
         </is>
@@ -841,7 +916,10 @@
       <c r="C28" t="n">
         <v>165712.862</v>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" t="n">
+        <v>165712.862</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>W</t>
         </is>
@@ -857,7 +935,10 @@
       <c r="C29" t="n">
         <v>1519.551</v>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" t="n">
+        <v>1519.551</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -873,7 +954,10 @@
       <c r="C30" t="n">
         <v>1519.551</v>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" t="n">
+        <v>1519.551</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -889,7 +973,10 @@
       <c r="C31" t="n">
         <v>88884.734</v>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" t="n">
+        <v>88884.734</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>W</t>
         </is>
@@ -905,7 +992,10 @@
       <c r="C32" t="n">
         <v>88884.734</v>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" t="n">
+        <v>88884.734</v>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t>W</t>
         </is>
@@ -921,7 +1011,10 @@
       <c r="C33" t="n">
         <v>15276.552</v>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" t="n">
+        <v>15276.552</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -937,7 +1030,10 @@
       <c r="C34" t="n">
         <v>1909.569</v>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" t="n">
+        <v>1909.569</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -953,7 +1049,10 @@
       <c r="C35" t="n">
         <v>243767.959</v>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" t="n">
+        <v>243767.959</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>W</t>
         </is>
@@ -969,7 +1068,10 @@
       <c r="C36" t="n">
         <v>30470.995</v>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" t="n">
+        <v>30470.995</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>W</t>
         </is>
@@ -985,7 +1087,10 @@
       <c r="C37" t="n">
         <v>247.599</v>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" t="n">
+        <v>247.599</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>N/m²</t>
         </is>
@@ -1000,6 +1105,7 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
@@ -1011,7 +1117,10 @@
       <c r="C39" t="n">
         <v>4.465</v>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" t="n">
+        <v>4.465</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>min</t>
         </is>
@@ -1027,7 +1136,10 @@
       <c r="C40" t="n">
         <v>23.836</v>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" t="n">
+        <v>23.836</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>min</t>
         </is>
@@ -1043,7 +1155,10 @@
       <c r="C41" t="n">
         <v>29.302</v>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" t="n">
+        <v>29.302</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>min</t>
         </is>
@@ -1058,6 +1173,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
@@ -1069,7 +1185,10 @@
       <c r="C43" t="n">
         <v>4062.799</v>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" t="n">
+        <v>4062.799</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>Wh</t>
         </is>
@@ -1085,7 +1204,10 @@
       <c r="C44" t="n">
         <v>12332.176</v>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" t="n">
+        <v>12332.176</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>Wh</t>
         </is>
@@ -1101,7 +1223,10 @@
       <c r="C45" t="n">
         <v>35311.566</v>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" t="n">
+        <v>35311.566</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>Wh</t>
         </is>
@@ -1117,7 +1242,10 @@
       <c r="C46" t="n">
         <v>51706.541</v>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" t="n">
+        <v>51706.541</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>Wh</t>
         </is>
@@ -1133,7 +1261,10 @@
       <c r="C47" t="n">
         <v>29628.245</v>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" t="n">
+        <v>29628.245</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>Wh</t>
         </is>
@@ -1149,7 +1280,10 @@
       <c r="C48" t="n">
         <v>81334.78599999999</v>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" t="n">
+        <v>81334.78599999999</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>Wh</t>
         </is>
@@ -1165,7 +1299,10 @@
       <c r="C49" t="n">
         <v>127085.603</v>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" t="n">
+        <v>127085.603</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>Wh</t>
         </is>
@@ -1181,7 +1318,10 @@
       <c r="C50" t="n">
         <v>45750.817</v>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" t="n">
+        <v>45750.817</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>Wh</t>
         </is>
@@ -1196,6 +1336,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr"/>
@@ -1207,7 +1348,10 @@
       <c r="C52" t="n">
         <v>15.858</v>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" t="n">
+        <v>15.858</v>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -1223,7 +1367,10 @@
       <c r="C53" t="n">
         <v>47.82</v>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" t="n">
+        <v>47.82</v>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -1239,7 +1386,10 @@
       <c r="C54" t="n">
         <v>82.61199999999999</v>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" t="n">
+        <v>82.61199999999999</v>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -1255,7 +1405,10 @@
       <c r="C55" t="n">
         <v>79.65000000000001</v>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" t="n">
+        <v>79.65000000000001</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -1271,7 +1424,10 @@
       <c r="C56" t="n">
         <v>199.462</v>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" t="n">
+        <v>199.462</v>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -1287,7 +1443,10 @@
       <c r="C57" t="n">
         <v>142.72</v>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" t="n">
+        <v>142.72</v>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -1303,7 +1462,10 @@
       <c r="C58" t="n">
         <v>79.303</v>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" t="n">
+        <v>79.303</v>
+      </c>
+      <c r="E58" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -1319,7 +1481,10 @@
       <c r="C59" t="n">
         <v>118.661</v>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D59" t="n">
+        <v>118.661</v>
+      </c>
+      <c r="E59" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -1335,7 +1500,10 @@
       <c r="C60" t="n">
         <v>392.8</v>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D60" t="n">
+        <v>392.8</v>
+      </c>
+      <c r="E60" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -1351,7 +1519,10 @@
       <c r="C61" t="n">
         <v>96.5</v>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -1367,7 +1538,10 @@
       <c r="C62" t="n">
         <v>317.714</v>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" t="n">
+        <v>317.714</v>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -1383,7 +1557,10 @@
       <c r="C63" t="n">
         <v>846.729</v>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D63" t="n">
+        <v>846.729</v>
+      </c>
+      <c r="E63" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -1399,7 +1576,10 @@
       <c r="C64" t="n">
         <v>1557.243</v>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" t="n">
+        <v>1557.243</v>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -1415,7 +1595,10 @@
       <c r="C65" t="n">
         <v>1557.243</v>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" t="n">
+        <v>1557.243</v>
+      </c>
+      <c r="E65" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -1431,7 +1614,10 @@
       <c r="C66" t="n">
         <v>0.204</v>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D66" t="n">
+        <v>0.204</v>
+      </c>
+      <c r="E66" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1447,7 +1633,10 @@
       <c r="C67" t="n">
         <v>0.544</v>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D67" t="n">
+        <v>0.544</v>
+      </c>
+      <c r="E67" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1462,6 +1651,7 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr"/>
@@ -1473,7 +1663,10 @@
       <c r="C69" t="n">
         <v>0.6909999999999999</v>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D69" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+      <c r="E69" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1489,7 +1682,10 @@
       <c r="C70" t="n">
         <v>678.995</v>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D70" t="n">
+        <v>678.995</v>
+      </c>
+      <c r="E70" t="inlineStr">
         <is>
           <t>RPM</t>
         </is>
@@ -1505,7 +1701,10 @@
       <c r="C71" t="n">
         <v>14.636</v>
       </c>
-      <c r="D71" t="inlineStr">
+      <c r="D71" t="n">
+        <v>14.636</v>
+      </c>
+      <c r="E71" t="inlineStr">
         <is>
           <t>dB</t>
         </is>
@@ -1521,7 +1720,10 @@
       <c r="C72" t="n">
         <v>1017.612</v>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D72" t="n">
+        <v>1017.612</v>
+      </c>
+      <c r="E72" t="inlineStr">
         <is>
           <t>RPM</t>
         </is>
@@ -1537,7 +1739,10 @@
       <c r="C73" t="n">
         <v>37.165</v>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D73" t="n">
+        <v>37.165</v>
+      </c>
+      <c r="E73" t="inlineStr">
         <is>
           <t>dB</t>
         </is>
@@ -1553,7 +1758,10 @@
       <c r="C74" t="n">
         <v>762.878</v>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D74" t="n">
+        <v>762.878</v>
+      </c>
+      <c r="E74" t="inlineStr">
         <is>
           <t>RPM</t>
         </is>
@@ -1569,7 +1777,10 @@
       <c r="C75" t="n">
         <v>69.833</v>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D75" t="n">
+        <v>69.833</v>
+      </c>
+      <c r="E75" t="inlineStr">
         <is>
           <t>dB</t>
         </is>
@@ -1584,6 +1795,7 @@
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr"/>
@@ -1595,7 +1807,10 @@
       <c r="C77" t="n">
         <v>1.918</v>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D77" t="n">
+        <v>1.918</v>
+      </c>
+      <c r="E77" t="inlineStr">
         <is>
           <t>1/h</t>
         </is>
@@ -1611,7 +1826,10 @@
       <c r="C78" t="n">
         <v>1.304</v>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="D78" t="n">
+        <v>1.304</v>
+      </c>
+      <c r="E78" t="inlineStr">
         <is>
           <t>1/h</t>
         </is>
@@ -1627,7 +1845,10 @@
       <c r="C79" t="n">
         <v>0.699</v>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D79" t="n">
+        <v>0.699</v>
+      </c>
+      <c r="E79" t="inlineStr">
         <is>
           <t>1/h</t>
         </is>
@@ -1643,7 +1864,10 @@
       <c r="C80" t="n">
         <v>0.833</v>
       </c>
-      <c r="D80" t="inlineStr">
+      <c r="D80" t="n">
+        <v>0.833</v>
+      </c>
+      <c r="E80" t="inlineStr">
         <is>
           <t>1/h</t>
         </is>
@@ -1659,7 +1883,10 @@
       <c r="C81" t="n">
         <v>0.407</v>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D81" t="n">
+        <v>0.407</v>
+      </c>
+      <c r="E81" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1675,7 +1902,10 @@
       <c r="C82" t="n">
         <v>5708.984</v>
       </c>
-      <c r="D82" t="inlineStr">
+      <c r="D82" t="n">
+        <v>5708.984</v>
+      </c>
+      <c r="E82" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1691,7 +1921,10 @@
       <c r="C83" t="n">
         <v>0.407</v>
       </c>
-      <c r="D83" t="inlineStr">
+      <c r="D83" t="n">
+        <v>0.407</v>
+      </c>
+      <c r="E83" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1706,6 +1939,7 @@
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr"/>
@@ -1717,7 +1951,10 @@
       <c r="C85" t="n">
         <v>24.412</v>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D85" t="n">
+        <v>24.412</v>
+      </c>
+      <c r="E85" t="inlineStr">
         <is>
           <t>min</t>
         </is>
@@ -1733,7 +1970,10 @@
       <c r="C86" t="n">
         <v>53.713</v>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D86" t="n">
+        <v>53.713</v>
+      </c>
+      <c r="E86" t="inlineStr">
         <is>
           <t>min</t>
         </is>
@@ -1749,7 +1989,10 @@
       <c r="C87" t="n">
         <v>1.833</v>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D87" t="n">
+        <v>1.833</v>
+      </c>
+      <c r="E87" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1765,7 +2008,10 @@
       <c r="C88" t="n">
         <v>8.936</v>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="D88" t="n">
+        <v>8.936</v>
+      </c>
+      <c r="E88" t="inlineStr">
         <is>
           <t>flights</t>
         </is>
@@ -1781,7 +2027,10 @@
       <c r="C89" t="n">
         <v>4.364</v>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D89" t="n">
+        <v>4.364</v>
+      </c>
+      <c r="E89" t="inlineStr">
         <is>
           <t>hours</t>
         </is>
@@ -1797,7 +2046,10 @@
       <c r="C90" t="n">
         <v>2323.443</v>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="D90" t="n">
+        <v>2323.443</v>
+      </c>
+      <c r="E90" t="inlineStr">
         <is>
           <t>flights</t>
         </is>
@@ -1813,7 +2065,10 @@
       <c r="C91" t="n">
         <v>1134.675</v>
       </c>
-      <c r="D91" t="inlineStr">
+      <c r="D91" t="n">
+        <v>1134.675</v>
+      </c>
+      <c r="E91" t="inlineStr">
         <is>
           <t>hours</t>
         </is>
@@ -1828,6 +2083,7 @@
       <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr"/>
@@ -1839,7 +2095,10 @@
       <c r="C93" t="n">
         <v>15822.158</v>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="D93" t="n">
+        <v>15822.158</v>
+      </c>
+      <c r="E93" t="inlineStr">
         <is>
           <t>kg CO2e</t>
         </is>
@@ -1855,7 +2114,10 @@
       <c r="C94" t="n">
         <v>6439.303</v>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="D94" t="n">
+        <v>6439.303</v>
+      </c>
+      <c r="E94" t="inlineStr">
         <is>
           <t>kg CO2e</t>
         </is>
@@ -1871,7 +2133,10 @@
       <c r="C95" t="n">
         <v>2.771</v>
       </c>
-      <c r="D95" t="inlineStr">
+      <c r="D95" t="n">
+        <v>2.771</v>
+      </c>
+      <c r="E95" t="inlineStr">
         <is>
           <t>kg CO2e</t>
         </is>
@@ -1887,7 +2152,10 @@
       <c r="C96" t="n">
         <v>19.595</v>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="D96" t="n">
+        <v>19.595</v>
+      </c>
+      <c r="E96" t="inlineStr">
         <is>
           <t>kg CO2e</t>
         </is>
@@ -1903,7 +2171,10 @@
       <c r="C97" t="n">
         <v>22.366</v>
       </c>
-      <c r="D97" t="inlineStr">
+      <c r="D97" t="n">
+        <v>22.366</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>kg CO2e</t>
         </is>
@@ -1919,7 +2190,10 @@
       <c r="C98" t="n">
         <v>51966.497</v>
       </c>
-      <c r="D98" t="inlineStr">
+      <c r="D98" t="n">
+        <v>51966.497</v>
+      </c>
+      <c r="E98" t="inlineStr">
         <is>
           <t>kg CO2e</t>
         </is>
@@ -1935,7 +2209,10 @@
       <c r="C99" t="n">
         <v>87.60899999999999</v>
       </c>
-      <c r="D99" t="inlineStr">
+      <c r="D99" t="n">
+        <v>87.60899999999999</v>
+      </c>
+      <c r="E99" t="inlineStr">
         <is>
           <t>%</t>
         </is>
@@ -1951,7 +2228,10 @@
       <c r="C100" t="n">
         <v>12.391</v>
       </c>
-      <c r="D100" t="inlineStr">
+      <c r="D100" t="n">
+        <v>12.391</v>
+      </c>
+      <c r="E100" t="inlineStr">
         <is>
           <t>%</t>
         </is>
@@ -1966,6 +2246,7 @@
       <c r="B101" t="inlineStr"/>
       <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr"/>
@@ -1977,7 +2258,10 @@
       <c r="C102" t="n">
         <v>4.998</v>
       </c>
-      <c r="D102" t="inlineStr">
+      <c r="D102" t="n">
+        <v>4.998</v>
+      </c>
+      <c r="E102" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -1993,7 +2277,10 @@
       <c r="C103" t="n">
         <v>16.967</v>
       </c>
-      <c r="D103" t="inlineStr">
+      <c r="D103" t="n">
+        <v>16.967</v>
+      </c>
+      <c r="E103" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2009,7 +2296,10 @@
       <c r="C104" t="n">
         <v>20.277</v>
       </c>
-      <c r="D104" t="inlineStr">
+      <c r="D104" t="n">
+        <v>20.277</v>
+      </c>
+      <c r="E104" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2025,7 +2315,10 @@
       <c r="C105" t="n">
         <v>16.116</v>
       </c>
-      <c r="D105" t="inlineStr">
+      <c r="D105" t="n">
+        <v>16.116</v>
+      </c>
+      <c r="E105" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2041,7 +2334,10 @@
       <c r="C106" t="n">
         <v>14614.844</v>
       </c>
-      <c r="D106" t="inlineStr">
+      <c r="D106" t="n">
+        <v>14614.844</v>
+      </c>
+      <c r="E106" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2057,7 +2353,10 @@
       <c r="C107" t="n">
         <v>2.56</v>
       </c>
-      <c r="D107" t="inlineStr">
+      <c r="D107" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="E107" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2073,7 +2372,10 @@
       <c r="C108" t="n">
         <v>18.676</v>
       </c>
-      <c r="D108" t="inlineStr">
+      <c r="D108" t="n">
+        <v>18.676</v>
+      </c>
+      <c r="E108" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2089,7 +2391,10 @@
       <c r="C109" t="n">
         <v>60.918</v>
       </c>
-      <c r="D109" t="inlineStr">
+      <c r="D109" t="n">
+        <v>60.918</v>
+      </c>
+      <c r="E109" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2105,7 +2410,10 @@
       <c r="C110" t="n">
         <v>45.326</v>
       </c>
-      <c r="D110" t="inlineStr">
+      <c r="D110" t="n">
+        <v>45.326</v>
+      </c>
+      <c r="E110" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2121,7 +2429,10 @@
       <c r="C111" t="n">
         <v>106.244</v>
       </c>
-      <c r="D111" t="inlineStr">
+      <c r="D111" t="n">
+        <v>106.244</v>
+      </c>
+      <c r="E111" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2137,7 +2448,10 @@
       <c r="C112" t="n">
         <v>23.355</v>
       </c>
-      <c r="D112" t="inlineStr">
+      <c r="D112" t="n">
+        <v>23.355</v>
+      </c>
+      <c r="E112" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2153,7 +2467,10 @@
       <c r="C113" t="n">
         <v>129.599</v>
       </c>
-      <c r="D113" t="inlineStr">
+      <c r="D113" t="n">
+        <v>129.599</v>
+      </c>
+      <c r="E113" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2169,7 +2486,10 @@
       <c r="C114" t="n">
         <v>0.463</v>
       </c>
-      <c r="D114" t="inlineStr">
+      <c r="D114" t="n">
+        <v>0.463</v>
+      </c>
+      <c r="E114" t="inlineStr">
         <is>
           <t>€/km</t>
         </is>
@@ -2185,7 +2505,10 @@
       <c r="C115" t="n">
         <v>1.106</v>
       </c>
-      <c r="D115" t="inlineStr">
+      <c r="D115" t="n">
+        <v>1.106</v>
+      </c>
+      <c r="E115" t="inlineStr">
         <is>
           <t>€/min</t>
         </is>
@@ -2200,6 +2523,7 @@
       <c r="B116" t="inlineStr"/>
       <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr"/>
+      <c r="E116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr"/>
@@ -2211,7 +2535,10 @@
       <c r="C117" t="n">
         <v>138.6</v>
       </c>
-      <c r="D117" t="inlineStr">
+      <c r="D117" t="n">
+        <v>138.6</v>
+      </c>
+      <c r="E117" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2227,7 +2554,10 @@
       <c r="C118" t="n">
         <v>376.992</v>
       </c>
-      <c r="D118" t="inlineStr">
+      <c r="D118" t="n">
+        <v>376.992</v>
+      </c>
+      <c r="E118" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2242,6 +2572,7 @@
       <c r="B119" t="inlineStr"/>
       <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr"/>
+      <c r="E119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr"/>
@@ -2253,7 +2584,10 @@
       <c r="C120" t="n">
         <v>247.393</v>
       </c>
-      <c r="D120" t="inlineStr">
+      <c r="D120" t="n">
+        <v>247.393</v>
+      </c>
+      <c r="E120" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2269,7 +2603,10 @@
       <c r="C121" t="n">
         <v>574803.964</v>
       </c>
-      <c r="D121" t="inlineStr">
+      <c r="D121" t="n">
+        <v>574803.964</v>
+      </c>
+      <c r="E121" t="inlineStr">
         <is>
           <t>€</t>
         </is>

</xml_diff>

<commit_message>
adjusted items are marked with --- IGNORE ---, deleted items are marked with deleted: and new files are marked with new file: in the list of changes below.
</commit_message>
<xml_diff>
--- a/src/results/GWP/optimized_results_GWP.xlsx
+++ b/src/results/GWP/optimized_results_GWP.xlsx
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.718</v>
+        <v>1.051</v>
       </c>
       <c r="D4" t="n">
         <v>1.718</v>
@@ -501,10 +501,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.569</v>
+        <v>0.832</v>
       </c>
       <c r="D5" t="n">
-        <v>1.569</v>
+        <v>1.568</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.567</v>
+        <v>1.371</v>
       </c>
       <c r="D6" t="n">
         <v>1.567</v>
@@ -588,10 +588,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>8.731999999999999</v>
+        <v>14.267</v>
       </c>
       <c r="D10" t="n">
-        <v>8.731999999999999</v>
+        <v>8.731</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.522</v>
+        <v>0.543</v>
       </c>
       <c r="D11" t="n">
         <v>0.522</v>
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.052</v>
+        <v>0.048</v>
       </c>
       <c r="D12" t="n">
         <v>0.052</v>
@@ -645,10 +645,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>10.015</v>
+        <v>11.327</v>
       </c>
       <c r="D13" t="n">
-        <v>10.015</v>
+        <v>10.014</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -664,10 +664,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1517.469</v>
+        <v>1298.44</v>
       </c>
       <c r="D14" t="n">
-        <v>1517.469</v>
+        <v>1517.503</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.919</v>
+        <v>0.975</v>
       </c>
       <c r="D15" t="n">
         <v>0.919</v>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.078</v>
+        <v>0.066</v>
       </c>
       <c r="D16" t="n">
         <v>0.078</v>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>11.754</v>
+        <v>14.725</v>
       </c>
       <c r="D17" t="n">
         <v>11.754</v>
@@ -740,10 +740,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1286.997</v>
+        <v>993.655</v>
       </c>
       <c r="D18" t="n">
-        <v>1286.997</v>
+        <v>1287.052</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -770,10 +770,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>42.955</v>
+        <v>52.965</v>
       </c>
       <c r="D20" t="n">
-        <v>42.955</v>
+        <v>42.953</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -789,10 +789,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>32.29</v>
+        <v>39.415</v>
       </c>
       <c r="D21" t="n">
-        <v>32.29</v>
+        <v>32.289</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -808,10 +808,10 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>31.976</v>
+        <v>39.032</v>
       </c>
       <c r="D22" t="n">
-        <v>31.976</v>
+        <v>31.975</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4.494</v>
+        <v>5.486</v>
       </c>
       <c r="D23" t="n">
         <v>4.494</v>
@@ -857,10 +857,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3413.082</v>
+        <v>3050.027</v>
       </c>
       <c r="D25" t="n">
-        <v>3413.082</v>
+        <v>3413.129</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -876,10 +876,10 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3413.082</v>
+        <v>3050.027</v>
       </c>
       <c r="D26" t="n">
-        <v>3413.082</v>
+        <v>3413.129</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -895,10 +895,10 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>165712.862</v>
+        <v>202145.183</v>
       </c>
       <c r="D27" t="n">
-        <v>165712.862</v>
+        <v>165713.351</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -914,10 +914,10 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>165712.862</v>
+        <v>202145.183</v>
       </c>
       <c r="D28" t="n">
-        <v>165712.862</v>
+        <v>165713.351</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -933,10 +933,10 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1519.551</v>
+        <v>1300.222</v>
       </c>
       <c r="D29" t="n">
-        <v>1519.551</v>
+        <v>1519.586</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -952,10 +952,10 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1519.551</v>
+        <v>1300.222</v>
       </c>
       <c r="D30" t="n">
-        <v>1519.551</v>
+        <v>1519.586</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>88884.734</v>
+        <v>97266.04399999999</v>
       </c>
       <c r="D31" t="n">
-        <v>88884.734</v>
+        <v>88883.826</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -990,10 +990,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>88884.734</v>
+        <v>97266.04399999999</v>
       </c>
       <c r="D32" t="n">
-        <v>88884.734</v>
+        <v>88883.826</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1009,10 +1009,10 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>15276.552</v>
+        <v>14775.642</v>
       </c>
       <c r="D33" t="n">
-        <v>15276.552</v>
+        <v>15276.496</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1028,10 +1028,10 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1909.569</v>
+        <v>1846.955</v>
       </c>
       <c r="D34" t="n">
-        <v>1909.569</v>
+        <v>1909.562</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1047,10 +1047,10 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>243767.959</v>
+        <v>265025.448</v>
       </c>
       <c r="D35" t="n">
-        <v>243767.959</v>
+        <v>243773.417</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1066,10 +1066,10 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>30470.995</v>
+        <v>33128.181</v>
       </c>
       <c r="D36" t="n">
-        <v>30470.995</v>
+        <v>30471.677</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1085,10 +1085,10 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>247.599</v>
+        <v>312.845</v>
       </c>
       <c r="D37" t="n">
-        <v>247.599</v>
+        <v>247.612</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>4.465</v>
+        <v>3.658</v>
       </c>
       <c r="D39" t="n">
         <v>4.465</v>
@@ -1134,10 +1134,10 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>23.836</v>
+        <v>19.331</v>
       </c>
       <c r="D40" t="n">
-        <v>23.836</v>
+        <v>23.837</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1153,10 +1153,10 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>29.302</v>
+        <v>23.989</v>
       </c>
       <c r="D41" t="n">
-        <v>29.302</v>
+        <v>29.303</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1183,10 +1183,10 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>4062.799</v>
+        <v>4417.091</v>
       </c>
       <c r="D43" t="n">
-        <v>4062.799</v>
+        <v>4062.89</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1202,10 +1202,10 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>12332.176</v>
+        <v>12324</v>
       </c>
       <c r="D44" t="n">
-        <v>12332.176</v>
+        <v>12332.726</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1221,10 +1221,10 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>35311.566</v>
+        <v>31338.246</v>
       </c>
       <c r="D45" t="n">
-        <v>35311.566</v>
+        <v>35312.759</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1240,10 +1240,10 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>51706.541</v>
+        <v>48079.337</v>
       </c>
       <c r="D46" t="n">
-        <v>51706.541</v>
+        <v>51708.375</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1259,10 +1259,10 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>29628.245</v>
+        <v>32422.015</v>
       </c>
       <c r="D47" t="n">
-        <v>29628.245</v>
+        <v>29627.942</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1278,10 +1278,10 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>81334.78599999999</v>
+        <v>80501.352</v>
       </c>
       <c r="D48" t="n">
-        <v>81334.78599999999</v>
+        <v>81336.317</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1297,10 +1297,10 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>127085.603</v>
+        <v>125783.363</v>
       </c>
       <c r="D49" t="n">
-        <v>127085.603</v>
+        <v>127087.995</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1316,10 +1316,10 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>45750.817</v>
+        <v>45282.011</v>
       </c>
       <c r="D50" t="n">
-        <v>45750.817</v>
+        <v>45751.678</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1346,10 +1346,10 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>15.858</v>
+        <v>12.808</v>
       </c>
       <c r="D52" t="n">
-        <v>15.858</v>
+        <v>15.857</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1365,10 +1365,10 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>47.82</v>
+        <v>48.238</v>
       </c>
       <c r="D53" t="n">
-        <v>47.82</v>
+        <v>47.819</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1384,10 +1384,10 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>82.61199999999999</v>
+        <v>40.392</v>
       </c>
       <c r="D54" t="n">
-        <v>82.61199999999999</v>
+        <v>82.60599999999999</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1403,10 +1403,10 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>79.65000000000001</v>
+        <v>91.41500000000001</v>
       </c>
       <c r="D55" t="n">
-        <v>79.65000000000001</v>
+        <v>79.648</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1422,10 +1422,10 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>199.462</v>
+        <v>219.387</v>
       </c>
       <c r="D56" t="n">
-        <v>199.462</v>
+        <v>199.465</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1441,10 +1441,10 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>142.72</v>
+        <v>115.269</v>
       </c>
       <c r="D57" t="n">
-        <v>142.72</v>
+        <v>142.714</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>79.303</v>
+        <v>77.45399999999999</v>
       </c>
       <c r="D58" t="n">
         <v>79.303</v>
@@ -1479,10 +1479,10 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>118.661</v>
+        <v>110.269</v>
       </c>
       <c r="D59" t="n">
-        <v>118.661</v>
+        <v>118.662</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1536,10 +1536,10 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>317.714</v>
+        <v>314.458</v>
       </c>
       <c r="D62" t="n">
-        <v>317.714</v>
+        <v>317.72</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1555,10 +1555,10 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>846.729</v>
+        <v>798.923</v>
       </c>
       <c r="D63" t="n">
-        <v>846.729</v>
+        <v>846.717</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1574,10 +1574,10 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1557.243</v>
+        <v>1506.182</v>
       </c>
       <c r="D64" t="n">
-        <v>1557.243</v>
+        <v>1557.237</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1593,10 +1593,10 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1557.243</v>
+        <v>1506.182</v>
       </c>
       <c r="D65" t="n">
-        <v>1557.243</v>
+        <v>1557.237</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>0.204</v>
+        <v>0.209</v>
       </c>
       <c r="D66" t="n">
         <v>0.204</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>0.544</v>
+        <v>0.53</v>
       </c>
       <c r="D67" t="n">
         <v>0.544</v>
@@ -1661,10 +1661,10 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0.6909999999999999</v>
+        <v>1.473</v>
       </c>
       <c r="D69" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1680,10 +1680,10 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>678.995</v>
+        <v>2231.571</v>
       </c>
       <c r="D70" t="n">
-        <v>678.995</v>
+        <v>679.119</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -1699,10 +1699,10 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>14.636</v>
+        <v>29.636</v>
       </c>
       <c r="D71" t="n">
-        <v>14.636</v>
+        <v>14.64</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1017.612</v>
+        <v>3417.856</v>
       </c>
       <c r="D72" t="n">
-        <v>1017.612</v>
+        <v>1017.793</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -1737,10 +1737,10 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>37.165</v>
+        <v>53.283</v>
       </c>
       <c r="D73" t="n">
-        <v>37.165</v>
+        <v>37.169</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -1756,10 +1756,10 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>762.878</v>
+        <v>980.109</v>
       </c>
       <c r="D74" t="n">
-        <v>762.878</v>
+        <v>762.919</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -1775,10 +1775,10 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>69.833</v>
+        <v>73.55500000000001</v>
       </c>
       <c r="D75" t="n">
-        <v>69.833</v>
+        <v>69.834</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1.918</v>
+        <v>2.107</v>
       </c>
       <c r="D77" t="n">
         <v>1.918</v>
@@ -1824,7 +1824,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1.304</v>
+        <v>1.607</v>
       </c>
       <c r="D78" t="n">
         <v>1.304</v>
@@ -1843,7 +1843,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>0.699</v>
+        <v>0.773</v>
       </c>
       <c r="D79" t="n">
         <v>0.699</v>
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>0.833</v>
+        <v>0.956</v>
       </c>
       <c r="D80" t="n">
         <v>0.833</v>
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0.407</v>
+        <v>0.382</v>
       </c>
       <c r="D81" t="n">
         <v>0.407</v>
@@ -1900,10 +1900,10 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>5708.984</v>
+        <v>4984.565</v>
       </c>
       <c r="D82" t="n">
-        <v>5708.984</v>
+        <v>5709.119</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>0.407</v>
+        <v>0.534</v>
       </c>
       <c r="D83" t="n">
         <v>0.407</v>
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>24.412</v>
+        <v>22.934</v>
       </c>
       <c r="D85" t="n">
         <v>24.412</v>
@@ -1968,10 +1968,10 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>53.713</v>
+        <v>46.924</v>
       </c>
       <c r="D86" t="n">
-        <v>53.713</v>
+        <v>53.715</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1.833</v>
+        <v>1.956</v>
       </c>
       <c r="D87" t="n">
         <v>1.833</v>
@@ -2006,7 +2006,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>8.936</v>
+        <v>10.229</v>
       </c>
       <c r="D88" t="n">
         <v>8.936</v>
@@ -2025,7 +2025,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>4.364</v>
+        <v>4.09</v>
       </c>
       <c r="D89" t="n">
         <v>4.364</v>
@@ -2044,10 +2044,10 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2323.443</v>
+        <v>2659.632</v>
       </c>
       <c r="D90" t="n">
-        <v>2323.443</v>
+        <v>2323.372</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2063,10 +2063,10 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1134.675</v>
+        <v>1063.384</v>
       </c>
       <c r="D91" t="n">
-        <v>1134.675</v>
+        <v>1134.688</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2093,10 +2093,10 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>15822.158</v>
+        <v>15660.029</v>
       </c>
       <c r="D93" t="n">
-        <v>15822.158</v>
+        <v>15822.455</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2112,10 +2112,10 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>6439.303</v>
+        <v>8355.778</v>
       </c>
       <c r="D94" t="n">
-        <v>6439.303</v>
+        <v>6439.075</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2131,7 +2131,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2.771</v>
+        <v>3.142</v>
       </c>
       <c r="D95" t="n">
         <v>2.771</v>
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>19.595</v>
+        <v>18.22</v>
       </c>
       <c r="D96" t="n">
         <v>19.595</v>
@@ -2169,10 +2169,10 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>22.366</v>
+        <v>21.362</v>
       </c>
       <c r="D97" t="n">
-        <v>22.366</v>
+        <v>22.367</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2188,10 +2188,10 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>51966.497</v>
+        <v>56814.665</v>
       </c>
       <c r="D98" t="n">
-        <v>51966.497</v>
+        <v>51966.493</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>87.60899999999999</v>
+        <v>85.29300000000001</v>
       </c>
       <c r="D99" t="n">
         <v>87.60899999999999</v>
@@ -2226,7 +2226,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>12.391</v>
+        <v>14.707</v>
       </c>
       <c r="D100" t="n">
         <v>12.391</v>
@@ -2256,10 +2256,10 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>4.998</v>
+        <v>4.648</v>
       </c>
       <c r="D102" t="n">
-        <v>4.998</v>
+        <v>4.999</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2275,7 +2275,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>16.967</v>
+        <v>16.64</v>
       </c>
       <c r="D103" t="n">
         <v>16.967</v>
@@ -2294,7 +2294,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>20.277</v>
+        <v>17.714</v>
       </c>
       <c r="D104" t="n">
         <v>20.277</v>
@@ -2313,10 +2313,10 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>16.116</v>
+        <v>13.194</v>
       </c>
       <c r="D105" t="n">
-        <v>16.116</v>
+        <v>16.117</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2332,10 +2332,10 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>14614.844</v>
+        <v>14465.087</v>
       </c>
       <c r="D106" t="n">
-        <v>14614.844</v>
+        <v>14615.119</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>2.56</v>
+        <v>2.902</v>
       </c>
       <c r="D107" t="n">
         <v>2.56</v>
@@ -2370,7 +2370,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>18.676</v>
+        <v>16.096</v>
       </c>
       <c r="D108" t="n">
         <v>18.676</v>
@@ -2389,10 +2389,10 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>60.918</v>
+        <v>55.098</v>
       </c>
       <c r="D109" t="n">
-        <v>60.918</v>
+        <v>60.919</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -2408,10 +2408,10 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>45.326</v>
+        <v>37.654</v>
       </c>
       <c r="D110" t="n">
-        <v>45.326</v>
+        <v>45.327</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -2427,10 +2427,10 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>106.244</v>
+        <v>92.752</v>
       </c>
       <c r="D111" t="n">
-        <v>106.244</v>
+        <v>106.246</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -2446,10 +2446,10 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>23.355</v>
+        <v>20.389</v>
       </c>
       <c r="D112" t="n">
-        <v>23.355</v>
+        <v>23.356</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -2465,10 +2465,10 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>129.599</v>
+        <v>113.141</v>
       </c>
       <c r="D113" t="n">
-        <v>129.599</v>
+        <v>129.602</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -2484,7 +2484,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>0.463</v>
+        <v>0.404</v>
       </c>
       <c r="D114" t="n">
         <v>0.463</v>
@@ -2503,7 +2503,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1.106</v>
+        <v>1.179</v>
       </c>
       <c r="D115" t="n">
         <v>1.106</v>
@@ -2582,10 +2582,10 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>247.393</v>
+        <v>263.851</v>
       </c>
       <c r="D120" t="n">
-        <v>247.393</v>
+        <v>247.39</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -2601,10 +2601,10 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>574803.964</v>
+        <v>701746.796</v>
       </c>
       <c r="D121" t="n">
-        <v>574803.964</v>
+        <v>574780.157</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -2685,13 +2685,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7.894</v>
+        <v>7.753</v>
       </c>
       <c r="C2" t="n">
         <v>64.235</v>
       </c>
       <c r="D2" t="n">
-        <v>8.775</v>
+        <v>8.617000000000001</v>
       </c>
       <c r="E2" t="n">
         <v>1.183</v>
@@ -2709,7 +2709,7 @@
         <v>1.911</v>
       </c>
       <c r="J2" t="n">
-        <v>5.492</v>
+        <v>5.227</v>
       </c>
     </row>
     <row r="3">
@@ -2719,13 +2719,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7.712</v>
+        <v>7.572</v>
       </c>
       <c r="C3" t="n">
         <v>64.235</v>
       </c>
       <c r="D3" t="n">
-        <v>8.775</v>
+        <v>8.617000000000001</v>
       </c>
       <c r="E3" t="n">
         <v>2.366</v>
@@ -2743,7 +2743,7 @@
         <v>1.547</v>
       </c>
       <c r="J3" t="n">
-        <v>5.527</v>
+        <v>5.264</v>
       </c>
     </row>
     <row r="4">
@@ -2753,13 +2753,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7.66</v>
+        <v>7.487</v>
       </c>
       <c r="C4" t="n">
         <v>50.909</v>
       </c>
       <c r="D4" t="n">
-        <v>9.242000000000001</v>
+        <v>9.074999999999999</v>
       </c>
       <c r="E4" t="n">
         <v>0.588</v>
@@ -2777,7 +2777,7 @@
         <v>16.8</v>
       </c>
       <c r="J4" t="n">
-        <v>4.029</v>
+        <v>3.678</v>
       </c>
     </row>
     <row r="5">
@@ -2787,13 +2787,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7.62</v>
+        <v>7.478</v>
       </c>
       <c r="C5" t="n">
         <v>64.235</v>
       </c>
       <c r="D5" t="n">
-        <v>8.775</v>
+        <v>8.617000000000001</v>
       </c>
       <c r="E5" t="n">
         <v>2.821</v>
@@ -2811,7 +2811,7 @@
         <v>2.093</v>
       </c>
       <c r="J5" t="n">
-        <v>5.474</v>
+        <v>5.208</v>
       </c>
     </row>
     <row r="6">
@@ -2821,13 +2821,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7.216</v>
+        <v>7.075</v>
       </c>
       <c r="C6" t="n">
         <v>105</v>
       </c>
       <c r="D6" t="n">
-        <v>7.346</v>
+        <v>7.217</v>
       </c>
       <c r="E6" t="n">
         <v>1.456</v>
@@ -2845,7 +2845,7 @@
         <v>6.72</v>
       </c>
       <c r="J6" t="n">
-        <v>5.019</v>
+        <v>4.726</v>
       </c>
     </row>
     <row r="7">
@@ -2855,13 +2855,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7.164</v>
+        <v>7.012</v>
       </c>
       <c r="C7" t="n">
         <v>64.235</v>
       </c>
       <c r="D7" t="n">
-        <v>8.775</v>
+        <v>8.617000000000001</v>
       </c>
       <c r="E7" t="n">
         <v>4.55</v>
@@ -2879,75 +2879,75 @@
         <v>7.371</v>
       </c>
       <c r="J7" t="n">
-        <v>4.955</v>
+        <v>4.659</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Train (50%)</t>
+          <t>Bicycle</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>7.036</v>
+        <v>6.999</v>
       </c>
       <c r="C8" t="n">
-        <v>50.909</v>
+        <v>285.957</v>
       </c>
       <c r="D8" t="n">
-        <v>9.242000000000001</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>1.008</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>9.504</v>
+        <v>10</v>
       </c>
       <c r="G8" t="n">
-        <v>9579.360000000001</v>
+        <v>-9955.456</v>
       </c>
       <c r="H8" t="n">
-        <v>7.396</v>
+        <v>10</v>
       </c>
       <c r="I8" t="n">
-        <v>33.768</v>
+        <v>-43.994</v>
       </c>
       <c r="J8" t="n">
-        <v>2.363</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Bicycle</t>
+          <t>Train (50%)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6.999</v>
+        <v>6.83</v>
       </c>
       <c r="C9" t="n">
-        <v>285.957</v>
+        <v>50.909</v>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>9.074999999999999</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>1.008</v>
       </c>
       <c r="F9" t="n">
-        <v>10</v>
+        <v>9.504</v>
       </c>
       <c r="G9" t="n">
-        <v>-9955.456</v>
+        <v>9579.360000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>10</v>
+        <v>7.396</v>
       </c>
       <c r="I9" t="n">
-        <v>-43.994</v>
+        <v>33.768</v>
       </c>
       <c r="J9" t="n">
-        <v>10</v>
+        <v>1.914</v>
       </c>
     </row>
     <row r="10">
@@ -2957,13 +2957,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6.889</v>
+        <v>6.739</v>
       </c>
       <c r="C10" t="n">
         <v>105</v>
       </c>
       <c r="D10" t="n">
-        <v>7.346</v>
+        <v>7.217</v>
       </c>
       <c r="E10" t="n">
         <v>2.464</v>
@@ -2981,7 +2981,7 @@
         <v>11.648</v>
       </c>
       <c r="J10" t="n">
-        <v>4.535</v>
+        <v>4.214</v>
       </c>
     </row>
     <row r="11">
@@ -2991,13 +2991,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6.868</v>
+        <v>6.713</v>
       </c>
       <c r="C11" t="n">
         <v>64.235</v>
       </c>
       <c r="D11" t="n">
-        <v>8.775</v>
+        <v>8.617000000000001</v>
       </c>
       <c r="E11" t="n">
         <v>5.915</v>
@@ -3015,7 +3015,7 @@
         <v>9.555</v>
       </c>
       <c r="J11" t="n">
-        <v>4.741</v>
+        <v>4.432</v>
       </c>
     </row>
     <row r="12">
@@ -3025,13 +3025,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.483</v>
+        <v>6.335</v>
       </c>
       <c r="C12" t="n">
         <v>64.235</v>
       </c>
       <c r="D12" t="n">
-        <v>8.775</v>
+        <v>8.617000000000001</v>
       </c>
       <c r="E12" t="n">
         <v>9.009</v>
@@ -3049,7 +3049,7 @@
         <v>5.824</v>
       </c>
       <c r="J12" t="n">
-        <v>5.107</v>
+        <v>4.82</v>
       </c>
     </row>
     <row r="13">
@@ -3059,13 +3059,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6.093</v>
+        <v>5.94</v>
       </c>
       <c r="C13" t="n">
         <v>64.235</v>
       </c>
       <c r="D13" t="n">
-        <v>8.775</v>
+        <v>8.617000000000001</v>
       </c>
       <c r="E13" t="n">
         <v>10.92</v>
@@ -3083,7 +3083,7 @@
         <v>8.19</v>
       </c>
       <c r="J13" t="n">
-        <v>4.875</v>
+        <v>4.574</v>
       </c>
     </row>
     <row r="14">
@@ -3093,13 +3093,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5.994</v>
+        <v>5.842</v>
       </c>
       <c r="C14" t="n">
         <v>64.235</v>
       </c>
       <c r="D14" t="n">
-        <v>8.775</v>
+        <v>8.617000000000001</v>
       </c>
       <c r="E14" t="n">
         <v>11.648</v>
@@ -3117,7 +3117,7 @@
         <v>7.553</v>
       </c>
       <c r="J14" t="n">
-        <v>4.938</v>
+        <v>4.64</v>
       </c>
     </row>
     <row r="15">
@@ -3127,31 +3127,31 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5.652</v>
+        <v>5.745</v>
       </c>
       <c r="C15" t="n">
-        <v>29.302</v>
+        <v>23.989</v>
       </c>
       <c r="D15" t="n">
         <v>10</v>
       </c>
       <c r="E15" t="n">
-        <v>8.223000000000001</v>
+        <v>7.854</v>
       </c>
       <c r="F15" t="n">
-        <v>5.956</v>
+        <v>6.138</v>
       </c>
       <c r="G15" t="n">
-        <v>19009.758</v>
+        <v>17676.227</v>
       </c>
       <c r="H15" t="n">
-        <v>6.138</v>
+        <v>6.316</v>
       </c>
       <c r="I15" t="n">
-        <v>47.647</v>
+        <v>41.596</v>
       </c>
       <c r="J15" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="16">
@@ -3161,13 +3161,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5.46</v>
+        <v>5.303</v>
       </c>
       <c r="C16" t="n">
         <v>64.235</v>
       </c>
       <c r="D16" t="n">
-        <v>8.775</v>
+        <v>8.617000000000001</v>
       </c>
       <c r="E16" t="n">
         <v>14.287</v>
@@ -3185,7 +3185,7 @@
         <v>10.647</v>
       </c>
       <c r="J16" t="n">
-        <v>4.634</v>
+        <v>4.318</v>
       </c>
     </row>
     <row r="17">
@@ -3195,13 +3195,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3.31</v>
+        <v>3.135</v>
       </c>
       <c r="C17" t="n">
         <v>179.595</v>
       </c>
       <c r="D17" t="n">
-        <v>4.73</v>
+        <v>4.654</v>
       </c>
       <c r="E17" t="n">
         <v>14.553</v>
@@ -3219,7 +3219,7 @@
         <v>33.81</v>
       </c>
       <c r="J17" t="n">
-        <v>2.359</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="18">
@@ -3229,13 +3229,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2.41</v>
+        <v>2.218</v>
       </c>
       <c r="C18" t="n">
         <v>179.595</v>
       </c>
       <c r="D18" t="n">
-        <v>4.73</v>
+        <v>4.654</v>
       </c>
       <c r="E18" t="n">
         <v>18.302</v>
@@ -3253,7 +3253,7 @@
         <v>42.556</v>
       </c>
       <c r="J18" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated README error and optic refinement of notebooks.
</commit_message>
<xml_diff>
--- a/src/results/GWP/optimized_results_GWP.xlsx
+++ b/src/results/GWP/optimized_results_GWP.xlsx
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.051</v>
+        <v>1.718</v>
       </c>
       <c r="D4" t="n">
         <v>1.718</v>
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.832</v>
+        <v>1.568</v>
       </c>
       <c r="D5" t="n">
         <v>1.568</v>
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.371</v>
+        <v>1.567</v>
       </c>
       <c r="D6" t="n">
         <v>1.567</v>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>14.267</v>
+        <v>8.731</v>
       </c>
       <c r="D10" t="n">
         <v>8.731</v>
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.543</v>
+        <v>0.522</v>
       </c>
       <c r="D11" t="n">
         <v>0.522</v>
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.048</v>
+        <v>0.052</v>
       </c>
       <c r="D12" t="n">
         <v>0.052</v>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>11.327</v>
+        <v>10.014</v>
       </c>
       <c r="D13" t="n">
         <v>10.014</v>
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1298.44</v>
+        <v>1517.503</v>
       </c>
       <c r="D14" t="n">
         <v>1517.503</v>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.975</v>
+        <v>0.919</v>
       </c>
       <c r="D15" t="n">
         <v>0.919</v>
@@ -702,7 +702,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.066</v>
+        <v>0.078</v>
       </c>
       <c r="D16" t="n">
         <v>0.078</v>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>14.725</v>
+        <v>11.754</v>
       </c>
       <c r="D17" t="n">
         <v>11.754</v>
@@ -740,7 +740,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>993.655</v>
+        <v>1287.052</v>
       </c>
       <c r="D18" t="n">
         <v>1287.052</v>
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>52.965</v>
+        <v>42.953</v>
       </c>
       <c r="D20" t="n">
         <v>42.953</v>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>39.415</v>
+        <v>32.289</v>
       </c>
       <c r="D21" t="n">
         <v>32.289</v>
@@ -808,7 +808,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>39.032</v>
+        <v>31.975</v>
       </c>
       <c r="D22" t="n">
         <v>31.975</v>
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>5.486</v>
+        <v>4.494</v>
       </c>
       <c r="D23" t="n">
         <v>4.494</v>
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3050.027</v>
+        <v>3413.129</v>
       </c>
       <c r="D25" t="n">
         <v>3413.129</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3050.027</v>
+        <v>3413.129</v>
       </c>
       <c r="D26" t="n">
         <v>3413.129</v>
@@ -895,7 +895,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>202145.183</v>
+        <v>165713.351</v>
       </c>
       <c r="D27" t="n">
         <v>165713.351</v>
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>202145.183</v>
+        <v>165713.351</v>
       </c>
       <c r="D28" t="n">
         <v>165713.351</v>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1300.222</v>
+        <v>1519.586</v>
       </c>
       <c r="D29" t="n">
         <v>1519.586</v>
@@ -952,7 +952,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1300.222</v>
+        <v>1519.586</v>
       </c>
       <c r="D30" t="n">
         <v>1519.586</v>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>97266.04399999999</v>
+        <v>88883.826</v>
       </c>
       <c r="D31" t="n">
         <v>88883.826</v>
@@ -990,7 +990,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>97266.04399999999</v>
+        <v>88883.826</v>
       </c>
       <c r="D32" t="n">
         <v>88883.826</v>
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>14775.642</v>
+        <v>15276.496</v>
       </c>
       <c r="D33" t="n">
         <v>15276.496</v>
@@ -1028,7 +1028,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1846.955</v>
+        <v>1909.562</v>
       </c>
       <c r="D34" t="n">
         <v>1909.562</v>
@@ -1047,7 +1047,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>265025.448</v>
+        <v>243773.417</v>
       </c>
       <c r="D35" t="n">
         <v>243773.417</v>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>33128.181</v>
+        <v>30471.677</v>
       </c>
       <c r="D36" t="n">
         <v>30471.677</v>
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>312.845</v>
+        <v>247.612</v>
       </c>
       <c r="D37" t="n">
         <v>247.612</v>
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3.658</v>
+        <v>4.465</v>
       </c>
       <c r="D39" t="n">
         <v>4.465</v>
@@ -1134,7 +1134,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>19.331</v>
+        <v>23.837</v>
       </c>
       <c r="D40" t="n">
         <v>23.837</v>
@@ -1153,7 +1153,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>23.989</v>
+        <v>29.303</v>
       </c>
       <c r="D41" t="n">
         <v>29.303</v>
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>4417.091</v>
+        <v>4062.89</v>
       </c>
       <c r="D43" t="n">
         <v>4062.89</v>
@@ -1202,7 +1202,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>12324</v>
+        <v>12332.726</v>
       </c>
       <c r="D44" t="n">
         <v>12332.726</v>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>31338.246</v>
+        <v>35312.759</v>
       </c>
       <c r="D45" t="n">
         <v>35312.759</v>
@@ -1240,7 +1240,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>48079.337</v>
+        <v>51708.375</v>
       </c>
       <c r="D46" t="n">
         <v>51708.375</v>
@@ -1259,7 +1259,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>32422.015</v>
+        <v>29627.942</v>
       </c>
       <c r="D47" t="n">
         <v>29627.942</v>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>80501.352</v>
+        <v>81336.317</v>
       </c>
       <c r="D48" t="n">
         <v>81336.317</v>
@@ -1297,7 +1297,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>125783.363</v>
+        <v>127087.995</v>
       </c>
       <c r="D49" t="n">
         <v>127087.995</v>
@@ -1316,7 +1316,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>45282.011</v>
+        <v>45751.678</v>
       </c>
       <c r="D50" t="n">
         <v>45751.678</v>
@@ -1346,7 +1346,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>12.808</v>
+        <v>15.857</v>
       </c>
       <c r="D52" t="n">
         <v>15.857</v>
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>48.238</v>
+        <v>47.819</v>
       </c>
       <c r="D53" t="n">
         <v>47.819</v>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>40.392</v>
+        <v>82.60599999999999</v>
       </c>
       <c r="D54" t="n">
         <v>82.60599999999999</v>
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>91.41500000000001</v>
+        <v>79.648</v>
       </c>
       <c r="D55" t="n">
         <v>79.648</v>
@@ -1422,7 +1422,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>219.387</v>
+        <v>199.465</v>
       </c>
       <c r="D56" t="n">
         <v>199.465</v>
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>115.269</v>
+        <v>142.714</v>
       </c>
       <c r="D57" t="n">
         <v>142.714</v>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>77.45399999999999</v>
+        <v>79.303</v>
       </c>
       <c r="D58" t="n">
         <v>79.303</v>
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>110.269</v>
+        <v>118.662</v>
       </c>
       <c r="D59" t="n">
         <v>118.662</v>
@@ -1536,7 +1536,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>314.458</v>
+        <v>317.72</v>
       </c>
       <c r="D62" t="n">
         <v>317.72</v>
@@ -1555,7 +1555,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>798.923</v>
+        <v>846.717</v>
       </c>
       <c r="D63" t="n">
         <v>846.717</v>
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1506.182</v>
+        <v>1557.237</v>
       </c>
       <c r="D64" t="n">
         <v>1557.237</v>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1506.182</v>
+        <v>1557.237</v>
       </c>
       <c r="D65" t="n">
         <v>1557.237</v>
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>0.209</v>
+        <v>0.204</v>
       </c>
       <c r="D66" t="n">
         <v>0.204</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>0.53</v>
+        <v>0.544</v>
       </c>
       <c r="D67" t="n">
         <v>0.544</v>
@@ -1661,7 +1661,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1.473</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="D69" t="n">
         <v>0.6919999999999999</v>
@@ -1680,7 +1680,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2231.571</v>
+        <v>679.119</v>
       </c>
       <c r="D70" t="n">
         <v>679.119</v>
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>29.636</v>
+        <v>14.64</v>
       </c>
       <c r="D71" t="n">
         <v>14.64</v>
@@ -1718,7 +1718,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>3417.856</v>
+        <v>1017.793</v>
       </c>
       <c r="D72" t="n">
         <v>1017.793</v>
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>53.283</v>
+        <v>37.169</v>
       </c>
       <c r="D73" t="n">
         <v>37.169</v>
@@ -1756,7 +1756,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>980.109</v>
+        <v>762.919</v>
       </c>
       <c r="D74" t="n">
         <v>762.919</v>
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>73.55500000000001</v>
+        <v>69.834</v>
       </c>
       <c r="D75" t="n">
         <v>69.834</v>
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2.107</v>
+        <v>1.918</v>
       </c>
       <c r="D77" t="n">
         <v>1.918</v>
@@ -1824,7 +1824,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1.607</v>
+        <v>1.304</v>
       </c>
       <c r="D78" t="n">
         <v>1.304</v>
@@ -1843,7 +1843,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>0.773</v>
+        <v>0.699</v>
       </c>
       <c r="D79" t="n">
         <v>0.699</v>
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>0.956</v>
+        <v>0.833</v>
       </c>
       <c r="D80" t="n">
         <v>0.833</v>
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0.382</v>
+        <v>0.407</v>
       </c>
       <c r="D81" t="n">
         <v>0.407</v>
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>4984.565</v>
+        <v>5709.119</v>
       </c>
       <c r="D82" t="n">
         <v>5709.119</v>
@@ -1919,7 +1919,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>0.534</v>
+        <v>0.407</v>
       </c>
       <c r="D83" t="n">
         <v>0.407</v>
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>22.934</v>
+        <v>24.412</v>
       </c>
       <c r="D85" t="n">
         <v>24.412</v>
@@ -1968,7 +1968,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>46.924</v>
+        <v>53.715</v>
       </c>
       <c r="D86" t="n">
         <v>53.715</v>
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1.956</v>
+        <v>1.833</v>
       </c>
       <c r="D87" t="n">
         <v>1.833</v>
@@ -2006,7 +2006,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>10.229</v>
+        <v>8.936</v>
       </c>
       <c r="D88" t="n">
         <v>8.936</v>
@@ -2025,7 +2025,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>4.09</v>
+        <v>4.364</v>
       </c>
       <c r="D89" t="n">
         <v>4.364</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2659.632</v>
+        <v>2323.372</v>
       </c>
       <c r="D90" t="n">
         <v>2323.372</v>
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1063.384</v>
+        <v>1134.688</v>
       </c>
       <c r="D91" t="n">
         <v>1134.688</v>
@@ -2093,7 +2093,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>15660.029</v>
+        <v>15822.455</v>
       </c>
       <c r="D93" t="n">
         <v>15822.455</v>
@@ -2112,7 +2112,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>8355.778</v>
+        <v>6439.075</v>
       </c>
       <c r="D94" t="n">
         <v>6439.075</v>
@@ -2131,7 +2131,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>3.142</v>
+        <v>2.771</v>
       </c>
       <c r="D95" t="n">
         <v>2.771</v>
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>18.22</v>
+        <v>19.595</v>
       </c>
       <c r="D96" t="n">
         <v>19.595</v>
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>21.362</v>
+        <v>22.367</v>
       </c>
       <c r="D97" t="n">
         <v>22.367</v>
@@ -2188,7 +2188,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>56814.665</v>
+        <v>51966.493</v>
       </c>
       <c r="D98" t="n">
         <v>51966.493</v>
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>85.29300000000001</v>
+        <v>87.60899999999999</v>
       </c>
       <c r="D99" t="n">
         <v>87.60899999999999</v>
@@ -2226,7 +2226,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>14.707</v>
+        <v>12.391</v>
       </c>
       <c r="D100" t="n">
         <v>12.391</v>
@@ -2256,7 +2256,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>4.648</v>
+        <v>4.999</v>
       </c>
       <c r="D102" t="n">
         <v>4.999</v>
@@ -2275,7 +2275,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>16.64</v>
+        <v>16.967</v>
       </c>
       <c r="D103" t="n">
         <v>16.967</v>
@@ -2294,7 +2294,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>17.714</v>
+        <v>20.277</v>
       </c>
       <c r="D104" t="n">
         <v>20.277</v>
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>13.194</v>
+        <v>16.117</v>
       </c>
       <c r="D105" t="n">
         <v>16.117</v>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>14465.087</v>
+        <v>14615.119</v>
       </c>
       <c r="D106" t="n">
         <v>14615.119</v>
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>2.902</v>
+        <v>2.56</v>
       </c>
       <c r="D107" t="n">
         <v>2.56</v>
@@ -2370,7 +2370,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>16.096</v>
+        <v>18.676</v>
       </c>
       <c r="D108" t="n">
         <v>18.676</v>
@@ -2389,7 +2389,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>55.098</v>
+        <v>60.919</v>
       </c>
       <c r="D109" t="n">
         <v>60.919</v>
@@ -2408,7 +2408,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>37.654</v>
+        <v>45.327</v>
       </c>
       <c r="D110" t="n">
         <v>45.327</v>
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>92.752</v>
+        <v>106.246</v>
       </c>
       <c r="D111" t="n">
         <v>106.246</v>
@@ -2446,7 +2446,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>20.389</v>
+        <v>23.356</v>
       </c>
       <c r="D112" t="n">
         <v>23.356</v>
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>113.141</v>
+        <v>129.602</v>
       </c>
       <c r="D113" t="n">
         <v>129.602</v>
@@ -2484,7 +2484,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>0.404</v>
+        <v>0.463</v>
       </c>
       <c r="D114" t="n">
         <v>0.463</v>
@@ -2503,7 +2503,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1.179</v>
+        <v>1.106</v>
       </c>
       <c r="D115" t="n">
         <v>1.106</v>
@@ -2582,7 +2582,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>263.851</v>
+        <v>247.39</v>
       </c>
       <c r="D120" t="n">
         <v>247.39</v>
@@ -2601,7 +2601,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>701746.796</v>
+        <v>574780.157</v>
       </c>
       <c r="D121" t="n">
         <v>574780.157</v>
@@ -2685,13 +2685,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7.753</v>
+        <v>7.894</v>
       </c>
       <c r="C2" t="n">
         <v>64.235</v>
       </c>
       <c r="D2" t="n">
-        <v>8.617000000000001</v>
+        <v>8.775</v>
       </c>
       <c r="E2" t="n">
         <v>1.183</v>
@@ -2709,7 +2709,7 @@
         <v>1.911</v>
       </c>
       <c r="J2" t="n">
-        <v>5.227</v>
+        <v>5.492</v>
       </c>
     </row>
     <row r="3">
@@ -2719,13 +2719,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7.572</v>
+        <v>7.712</v>
       </c>
       <c r="C3" t="n">
         <v>64.235</v>
       </c>
       <c r="D3" t="n">
-        <v>8.617000000000001</v>
+        <v>8.775</v>
       </c>
       <c r="E3" t="n">
         <v>2.366</v>
@@ -2743,7 +2743,7 @@
         <v>1.547</v>
       </c>
       <c r="J3" t="n">
-        <v>5.264</v>
+        <v>5.527</v>
       </c>
     </row>
     <row r="4">
@@ -2753,13 +2753,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7.487</v>
+        <v>7.66</v>
       </c>
       <c r="C4" t="n">
         <v>50.909</v>
       </c>
       <c r="D4" t="n">
-        <v>9.074999999999999</v>
+        <v>9.242000000000001</v>
       </c>
       <c r="E4" t="n">
         <v>0.588</v>
@@ -2777,7 +2777,7 @@
         <v>16.8</v>
       </c>
       <c r="J4" t="n">
-        <v>3.678</v>
+        <v>4.03</v>
       </c>
     </row>
     <row r="5">
@@ -2787,13 +2787,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7.478</v>
+        <v>7.62</v>
       </c>
       <c r="C5" t="n">
         <v>64.235</v>
       </c>
       <c r="D5" t="n">
-        <v>8.617000000000001</v>
+        <v>8.775</v>
       </c>
       <c r="E5" t="n">
         <v>2.821</v>
@@ -2811,7 +2811,7 @@
         <v>2.093</v>
       </c>
       <c r="J5" t="n">
-        <v>5.208</v>
+        <v>5.474</v>
       </c>
     </row>
     <row r="6">
@@ -2821,13 +2821,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7.075</v>
+        <v>7.216</v>
       </c>
       <c r="C6" t="n">
         <v>105</v>
       </c>
       <c r="D6" t="n">
-        <v>7.217</v>
+        <v>7.346</v>
       </c>
       <c r="E6" t="n">
         <v>1.456</v>
@@ -2845,7 +2845,7 @@
         <v>6.72</v>
       </c>
       <c r="J6" t="n">
-        <v>4.726</v>
+        <v>5.019</v>
       </c>
     </row>
     <row r="7">
@@ -2855,13 +2855,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7.012</v>
+        <v>7.164</v>
       </c>
       <c r="C7" t="n">
         <v>64.235</v>
       </c>
       <c r="D7" t="n">
-        <v>8.617000000000001</v>
+        <v>8.775</v>
       </c>
       <c r="E7" t="n">
         <v>4.55</v>
@@ -2879,75 +2879,75 @@
         <v>7.371</v>
       </c>
       <c r="J7" t="n">
-        <v>4.659</v>
+        <v>4.956</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bicycle</t>
+          <t>Train (50%)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6.999</v>
+        <v>7.036</v>
       </c>
       <c r="C8" t="n">
-        <v>285.957</v>
+        <v>50.909</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>9.242000000000001</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>1.008</v>
       </c>
       <c r="F8" t="n">
-        <v>10</v>
+        <v>9.504</v>
       </c>
       <c r="G8" t="n">
-        <v>-9955.456</v>
+        <v>9579.360000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>10</v>
+        <v>7.396</v>
       </c>
       <c r="I8" t="n">
-        <v>-43.994</v>
+        <v>33.768</v>
       </c>
       <c r="J8" t="n">
-        <v>10</v>
+        <v>2.363</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Train (50%)</t>
+          <t>Bicycle</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6.83</v>
+        <v>6.999</v>
       </c>
       <c r="C9" t="n">
-        <v>50.909</v>
+        <v>285.957</v>
       </c>
       <c r="D9" t="n">
-        <v>9.074999999999999</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>1.008</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>9.504</v>
+        <v>10</v>
       </c>
       <c r="G9" t="n">
-        <v>9579.360000000001</v>
+        <v>-9955.456</v>
       </c>
       <c r="H9" t="n">
-        <v>7.396</v>
+        <v>10</v>
       </c>
       <c r="I9" t="n">
-        <v>33.768</v>
+        <v>-43.994</v>
       </c>
       <c r="J9" t="n">
-        <v>1.914</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -2957,13 +2957,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6.739</v>
+        <v>6.889</v>
       </c>
       <c r="C10" t="n">
         <v>105</v>
       </c>
       <c r="D10" t="n">
-        <v>7.217</v>
+        <v>7.346</v>
       </c>
       <c r="E10" t="n">
         <v>2.464</v>
@@ -2981,7 +2981,7 @@
         <v>11.648</v>
       </c>
       <c r="J10" t="n">
-        <v>4.214</v>
+        <v>4.535</v>
       </c>
     </row>
     <row r="11">
@@ -2991,13 +2991,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6.713</v>
+        <v>6.868</v>
       </c>
       <c r="C11" t="n">
         <v>64.235</v>
       </c>
       <c r="D11" t="n">
-        <v>8.617000000000001</v>
+        <v>8.775</v>
       </c>
       <c r="E11" t="n">
         <v>5.915</v>
@@ -3015,7 +3015,7 @@
         <v>9.555</v>
       </c>
       <c r="J11" t="n">
-        <v>4.432</v>
+        <v>4.741</v>
       </c>
     </row>
     <row r="12">
@@ -3025,13 +3025,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.335</v>
+        <v>6.483</v>
       </c>
       <c r="C12" t="n">
         <v>64.235</v>
       </c>
       <c r="D12" t="n">
-        <v>8.617000000000001</v>
+        <v>8.775</v>
       </c>
       <c r="E12" t="n">
         <v>9.009</v>
@@ -3049,7 +3049,7 @@
         <v>5.824</v>
       </c>
       <c r="J12" t="n">
-        <v>4.82</v>
+        <v>5.107</v>
       </c>
     </row>
     <row r="13">
@@ -3059,13 +3059,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5.94</v>
+        <v>6.093</v>
       </c>
       <c r="C13" t="n">
         <v>64.235</v>
       </c>
       <c r="D13" t="n">
-        <v>8.617000000000001</v>
+        <v>8.775</v>
       </c>
       <c r="E13" t="n">
         <v>10.92</v>
@@ -3083,7 +3083,7 @@
         <v>8.19</v>
       </c>
       <c r="J13" t="n">
-        <v>4.574</v>
+        <v>4.875</v>
       </c>
     </row>
     <row r="14">
@@ -3093,13 +3093,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5.842</v>
+        <v>5.994</v>
       </c>
       <c r="C14" t="n">
         <v>64.235</v>
       </c>
       <c r="D14" t="n">
-        <v>8.617000000000001</v>
+        <v>8.775</v>
       </c>
       <c r="E14" t="n">
         <v>11.648</v>
@@ -3117,7 +3117,7 @@
         <v>7.553</v>
       </c>
       <c r="J14" t="n">
-        <v>4.64</v>
+        <v>4.938</v>
       </c>
     </row>
     <row r="15">
@@ -3127,31 +3127,31 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5.745</v>
+        <v>5.651</v>
       </c>
       <c r="C15" t="n">
-        <v>23.989</v>
+        <v>29.303</v>
       </c>
       <c r="D15" t="n">
         <v>10</v>
       </c>
       <c r="E15" t="n">
-        <v>7.854</v>
+        <v>8.223000000000001</v>
       </c>
       <c r="F15" t="n">
+        <v>5.956</v>
+      </c>
+      <c r="G15" t="n">
+        <v>19010.432</v>
+      </c>
+      <c r="H15" t="n">
         <v>6.138</v>
       </c>
-      <c r="G15" t="n">
-        <v>17676.227</v>
-      </c>
-      <c r="H15" t="n">
-        <v>6.316</v>
-      </c>
       <c r="I15" t="n">
-        <v>41.596</v>
+        <v>47.648</v>
       </c>
       <c r="J15" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -3161,13 +3161,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5.303</v>
+        <v>5.46</v>
       </c>
       <c r="C16" t="n">
         <v>64.235</v>
       </c>
       <c r="D16" t="n">
-        <v>8.617000000000001</v>
+        <v>8.775</v>
       </c>
       <c r="E16" t="n">
         <v>14.287</v>
@@ -3185,7 +3185,7 @@
         <v>10.647</v>
       </c>
       <c r="J16" t="n">
-        <v>4.318</v>
+        <v>4.634</v>
       </c>
     </row>
     <row r="17">
@@ -3195,13 +3195,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3.135</v>
+        <v>3.31</v>
       </c>
       <c r="C17" t="n">
         <v>179.595</v>
       </c>
       <c r="D17" t="n">
-        <v>4.654</v>
+        <v>4.73</v>
       </c>
       <c r="E17" t="n">
         <v>14.553</v>
@@ -3219,7 +3219,7 @@
         <v>33.81</v>
       </c>
       <c r="J17" t="n">
-        <v>1.91</v>
+        <v>2.359</v>
       </c>
     </row>
     <row r="18">
@@ -3229,13 +3229,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2.218</v>
+        <v>2.41</v>
       </c>
       <c r="C18" t="n">
         <v>179.595</v>
       </c>
       <c r="D18" t="n">
-        <v>4.654</v>
+        <v>4.73</v>
       </c>
       <c r="E18" t="n">
         <v>18.302</v>
@@ -3253,7 +3253,7 @@
         <v>42.556</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated README.md and file naming
</commit_message>
<xml_diff>
--- a/src/results/GWP/optimized_results_GWP.xlsx
+++ b/src/results/GWP/optimized_results_GWP.xlsx
@@ -463,10 +463,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>12.738</v>
+        <v>15</v>
       </c>
       <c r="D3" t="n">
-        <v>6.868</v>
+        <v>15</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -501,10 +501,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.333</v>
+        <v>1.353</v>
       </c>
       <c r="D5" t="n">
-        <v>1.135</v>
+        <v>1.353</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -520,10 +520,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.687</v>
+        <v>1.677</v>
       </c>
       <c r="D6" t="n">
-        <v>0.894</v>
+        <v>1.677</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -558,10 +558,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.869</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>3.746</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>12.738</v>
+        <v>15</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.539</v>
+        <v>0.545</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.049</v>
+        <v>0.048</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>11.044</v>
+        <v>11.448</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1392.272</v>
+        <v>1321.021</v>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.964</v>
+        <v>0.98</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.065</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>14.025</v>
+        <v>15.035</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1090.835</v>
+        <v>1000.586</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>60.498</v>
+        <v>54.981</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>45.11</v>
+        <v>40.883</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>44.671</v>
+        <v>40.485</v>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>6.278</v>
+        <v>5.69</v>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3241.039</v>
+        <v>3114.897</v>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
@@ -848,7 +848,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3241.039</v>
+        <v>3114.897</v>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>211252.908</v>
+        <v>186154.231</v>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>211252.908</v>
+        <v>186154.231</v>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1394.182</v>
+        <v>1322.834</v>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1394.182</v>
+        <v>1322.834</v>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>113245.167</v>
+        <v>97939.541</v>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>113245.167</v>
+        <v>97939.541</v>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>15449.852</v>
+        <v>15191.953</v>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
@@ -984,7 +984,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1931.231</v>
+        <v>1898.994</v>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>230282.037</v>
+        <v>225815.166</v>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>28785.255</v>
+        <v>28226.896</v>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>216.032</v>
+        <v>214.845</v>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3.196</v>
+        <v>3.527</v>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>16.924</v>
+        <v>18.623</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>21.121</v>
+        <v>23.149</v>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
@@ -1125,7 +1125,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>3838.034</v>
+        <v>3763.586</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
@@ -1142,7 +1142,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>11253.465</v>
+        <v>10941.742</v>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>31943.46</v>
+        <v>30398.053</v>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
@@ -1176,7 +1176,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>47034.959</v>
+        <v>45103.381</v>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>37748.389</v>
+        <v>32646.514</v>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
@@ -1210,7 +1210,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>84783.348</v>
+        <v>77749.895</v>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>132473.981</v>
+        <v>121484.21</v>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>47690.633</v>
+        <v>43734.316</v>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
@@ -1272,7 +1272,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>16.86</v>
+        <v>16.781</v>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>51.554</v>
+        <v>49.834</v>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
@@ -1306,7 +1306,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>72.203</v>
+        <v>72.32299999999999</v>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
@@ -1323,7 +1323,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>101.397</v>
+        <v>94.41</v>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
@@ -1340,7 +1340,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>206.919</v>
+        <v>197.665</v>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>151.736</v>
+        <v>151.027</v>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>79.571</v>
+        <v>78.992</v>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
@@ -1391,7 +1391,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>91.04300000000001</v>
+        <v>111.357</v>
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
@@ -1442,7 +1442,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>331.185</v>
+        <v>303.711</v>
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
@@ -1459,7 +1459,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>850.924</v>
+        <v>852.109</v>
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
@@ -1476,7 +1476,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1574.908</v>
+        <v>1548.619</v>
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1574.908</v>
+        <v>1548.619</v>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
@@ -1510,7 +1510,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>0.21</v>
+        <v>0.196</v>
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
@@ -1555,7 +1555,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0.466</v>
+        <v>0.529</v>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>900.737</v>
+        <v>851.502</v>
       </c>
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
@@ -1606,7 +1606,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1373.348</v>
+        <v>1306.636</v>
       </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
@@ -1623,7 +1623,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>35.891</v>
+        <v>36.218</v>
       </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr">
@@ -1640,7 +1640,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>661.873</v>
+        <v>663.8</v>
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>67.628</v>
+        <v>67.464</v>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
@@ -1685,7 +1685,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1.738</v>
+        <v>1.859</v>
       </c>
       <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
@@ -1702,7 +1702,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1.595</v>
+        <v>1.532</v>
       </c>
       <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
@@ -1719,7 +1719,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>0.855</v>
+        <v>0.806</v>
       </c>
       <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1.009</v>
+        <v>0.962</v>
       </c>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0.355</v>
+        <v>0.371</v>
       </c>
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
@@ -1770,7 +1770,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2257.33</v>
+        <v>4983.123</v>
       </c>
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1.7</v>
+        <v>0.551</v>
       </c>
       <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr">
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>11.4</v>
+        <v>22.276</v>
       </c>
       <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
@@ -1832,7 +1832,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>32.521</v>
+        <v>45.425</v>
       </c>
       <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1.54</v>
+        <v>1.962</v>
       </c>
       <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>14.76</v>
+        <v>10.567</v>
       </c>
       <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr">
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>5.196</v>
+        <v>4.077</v>
       </c>
       <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>3837.516</v>
+        <v>2747.363</v>
       </c>
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1350.845</v>
+        <v>1059.988</v>
       </c>
       <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr">
@@ -1945,7 +1945,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>16493.011</v>
+        <v>15124.784</v>
       </c>
       <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr">
@@ -1962,7 +1962,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>28038.514</v>
+        <v>8338.800999999999</v>
       </c>
       <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr">
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>7.306</v>
+        <v>3.035</v>
       </c>
       <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
@@ -1996,7 +1996,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>17.824</v>
+        <v>17.092</v>
       </c>
       <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
@@ -2013,7 +2013,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>25.131</v>
+        <v>20.128</v>
       </c>
       <c r="D97" t="inlineStr"/>
       <c r="E97" t="inlineStr">
@@ -2030,7 +2030,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>96439.811</v>
+        <v>55297.762</v>
       </c>
       <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>70.926</v>
+        <v>84.92</v>
       </c>
       <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr">
@@ -2064,7 +2064,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>29.074</v>
+        <v>15.08</v>
       </c>
       <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr">
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>4.547</v>
+        <v>4.36</v>
       </c>
       <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr">
@@ -2109,7 +2109,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>17.079</v>
+        <v>16.912</v>
       </c>
       <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr">
@@ -2126,7 +2126,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>12.277</v>
+        <v>17.148</v>
       </c>
       <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr">
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>11.616</v>
+        <v>12.732</v>
       </c>
       <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr">
@@ -2160,7 +2160,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>15234.508</v>
+        <v>13970.684</v>
       </c>
       <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr">
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>6.749</v>
+        <v>2.804</v>
       </c>
       <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr">
@@ -2194,7 +2194,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>18.365</v>
+        <v>15.536</v>
       </c>
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr">
@@ -2211,7 +2211,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>52.268</v>
+        <v>53.956</v>
       </c>
       <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr">
@@ -2228,7 +2228,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>28.491</v>
+        <v>38.702</v>
       </c>
       <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr">
@@ -2245,7 +2245,7 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>80.758</v>
+        <v>92.658</v>
       </c>
       <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>17.753</v>
+        <v>20.369</v>
       </c>
       <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr">
@@ -2279,7 +2279,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>98.511</v>
+        <v>113.027</v>
       </c>
       <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr">
@@ -2296,7 +2296,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>0.352</v>
+        <v>0.404</v>
       </c>
       <c r="D114" t="inlineStr"/>
       <c r="E114" t="inlineStr">
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1.166</v>
+        <v>1.221</v>
       </c>
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr">
@@ -2386,7 +2386,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>278.481</v>
+        <v>263.965</v>
       </c>
       <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr">
@@ -2403,7 +2403,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1068675.446</v>
+        <v>725208.77</v>
       </c>
       <c r="D121" t="inlineStr"/>
       <c r="E121" t="inlineStr">
@@ -2485,13 +2485,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7.726</v>
+        <v>7.745</v>
       </c>
       <c r="C2" t="n">
         <v>64.235</v>
       </c>
       <c r="D2" t="n">
-        <v>8.535</v>
+        <v>8.593</v>
       </c>
       <c r="E2" t="n">
         <v>1.183</v>
@@ -2519,13 +2519,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7.544</v>
+        <v>7.564</v>
       </c>
       <c r="C3" t="n">
         <v>64.235</v>
       </c>
       <c r="D3" t="n">
-        <v>8.535</v>
+        <v>8.593</v>
       </c>
       <c r="E3" t="n">
         <v>2.366</v>
@@ -2553,13 +2553,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7.458</v>
+        <v>7.479</v>
       </c>
       <c r="C4" t="n">
         <v>50.909</v>
       </c>
       <c r="D4" t="n">
-        <v>8.988</v>
+        <v>9.048999999999999</v>
       </c>
       <c r="E4" t="n">
         <v>0.588</v>
@@ -2587,13 +2587,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7.451</v>
+        <v>7.47</v>
       </c>
       <c r="C5" t="n">
         <v>64.235</v>
       </c>
       <c r="D5" t="n">
-        <v>8.535</v>
+        <v>8.593</v>
       </c>
       <c r="E5" t="n">
         <v>2.821</v>
@@ -2621,13 +2621,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7.053</v>
+        <v>7.068</v>
       </c>
       <c r="C6" t="n">
         <v>105</v>
       </c>
       <c r="D6" t="n">
-        <v>7.15</v>
+        <v>7.197</v>
       </c>
       <c r="E6" t="n">
         <v>1.456</v>
@@ -2651,69 +2651,69 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bicycle</t>
+          <t>Electric Vehicle (26%)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6.999</v>
+        <v>7.004</v>
       </c>
       <c r="C7" t="n">
-        <v>285.957</v>
+        <v>64.235</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>8.593</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>4.55</v>
       </c>
       <c r="F7" t="n">
-        <v>10</v>
+        <v>7.762</v>
       </c>
       <c r="G7" t="n">
-        <v>-9955.456</v>
+        <v>12089.35</v>
       </c>
       <c r="H7" t="n">
-        <v>10</v>
+        <v>7.061</v>
       </c>
       <c r="I7" t="n">
-        <v>-43.994</v>
+        <v>7.371</v>
       </c>
       <c r="J7" t="n">
-        <v>10</v>
+        <v>4.659</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Electric Vehicle (26%)</t>
+          <t>Bicycle</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6.985</v>
+        <v>6.999</v>
       </c>
       <c r="C8" t="n">
-        <v>64.235</v>
+        <v>285.957</v>
       </c>
       <c r="D8" t="n">
-        <v>8.535</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>4.55</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>7.762</v>
+        <v>10</v>
       </c>
       <c r="G8" t="n">
-        <v>12089.35</v>
+        <v>-9955.456</v>
       </c>
       <c r="H8" t="n">
-        <v>7.061</v>
+        <v>10</v>
       </c>
       <c r="I8" t="n">
-        <v>7.371</v>
+        <v>-43.994</v>
       </c>
       <c r="J8" t="n">
-        <v>4.659</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -2723,13 +2723,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6.801</v>
+        <v>6.822</v>
       </c>
       <c r="C9" t="n">
         <v>50.909</v>
       </c>
       <c r="D9" t="n">
-        <v>8.988</v>
+        <v>9.048999999999999</v>
       </c>
       <c r="E9" t="n">
         <v>1.008</v>
@@ -2757,13 +2757,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6.717</v>
+        <v>6.732</v>
       </c>
       <c r="C10" t="n">
         <v>105</v>
       </c>
       <c r="D10" t="n">
-        <v>7.15</v>
+        <v>7.197</v>
       </c>
       <c r="E10" t="n">
         <v>2.464</v>
@@ -2791,13 +2791,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6.685</v>
+        <v>6.705</v>
       </c>
       <c r="C11" t="n">
         <v>64.235</v>
       </c>
       <c r="D11" t="n">
-        <v>8.535</v>
+        <v>8.593</v>
       </c>
       <c r="E11" t="n">
         <v>5.915</v>
@@ -2825,13 +2825,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.307</v>
+        <v>6.327</v>
       </c>
       <c r="C12" t="n">
         <v>64.235</v>
       </c>
       <c r="D12" t="n">
-        <v>8.535</v>
+        <v>8.593</v>
       </c>
       <c r="E12" t="n">
         <v>9.009</v>
@@ -2859,13 +2859,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5.912</v>
+        <v>5.932</v>
       </c>
       <c r="C13" t="n">
         <v>64.235</v>
       </c>
       <c r="D13" t="n">
-        <v>8.535</v>
+        <v>8.593</v>
       </c>
       <c r="E13" t="n">
         <v>10.92</v>
@@ -2893,13 +2893,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5.815</v>
+        <v>5.834</v>
       </c>
       <c r="C14" t="n">
         <v>64.235</v>
       </c>
       <c r="D14" t="n">
-        <v>8.535</v>
+        <v>8.593</v>
       </c>
       <c r="E14" t="n">
         <v>11.648</v>
@@ -2927,31 +2927,31 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5.705</v>
+        <v>5.821</v>
       </c>
       <c r="C15" t="n">
-        <v>21.121</v>
+        <v>23.149</v>
       </c>
       <c r="D15" t="n">
         <v>10</v>
       </c>
       <c r="E15" t="n">
-        <v>9.239000000000001</v>
+        <v>7.4</v>
       </c>
       <c r="F15" t="n">
-        <v>5.456</v>
+        <v>6.361</v>
       </c>
       <c r="G15" t="n">
-        <v>17292.264</v>
+        <v>16582.125</v>
       </c>
       <c r="H15" t="n">
-        <v>6.367</v>
+        <v>6.462</v>
       </c>
       <c r="I15" t="n">
-        <v>36.217</v>
+        <v>41.554</v>
       </c>
       <c r="J15" t="n">
-        <v>1.659</v>
+        <v>1.104</v>
       </c>
     </row>
     <row r="16">
@@ -2961,13 +2961,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5.275</v>
+        <v>5.295</v>
       </c>
       <c r="C16" t="n">
         <v>64.235</v>
       </c>
       <c r="D16" t="n">
-        <v>8.535</v>
+        <v>8.593</v>
       </c>
       <c r="E16" t="n">
         <v>14.287</v>
@@ -2995,13 +2995,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3.122</v>
+        <v>3.131</v>
       </c>
       <c r="C17" t="n">
         <v>179.595</v>
       </c>
       <c r="D17" t="n">
-        <v>4.615</v>
+        <v>4.642</v>
       </c>
       <c r="E17" t="n">
         <v>14.553</v>
@@ -3029,13 +3029,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2.205</v>
+        <v>2.214</v>
       </c>
       <c r="C18" t="n">
         <v>179.595</v>
       </c>
       <c r="D18" t="n">
-        <v>4.615</v>
+        <v>4.642</v>
       </c>
       <c r="E18" t="n">
         <v>18.302</v>

</xml_diff>

<commit_message>
updated formatting in README.md
</commit_message>
<xml_diff>
--- a/src/results/GWP/optimized_results_GWP.xlsx
+++ b/src/results/GWP/optimized_results_GWP.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,10 +463,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>15</v>
+        <v>11.584</v>
       </c>
       <c r="D3" t="n">
-        <v>15</v>
+        <v>9.877000000000001</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -501,10 +501,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.353</v>
+        <v>1.022</v>
       </c>
       <c r="D5" t="n">
-        <v>1.353</v>
+        <v>0.85</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -520,10 +520,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.677</v>
+        <v>1.568</v>
       </c>
       <c r="D6" t="n">
-        <v>1.677</v>
+        <v>1.395</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -558,10 +558,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>1.627</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>2.023</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>15</v>
+        <v>11.584</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.545</v>
+        <v>0.535</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.048</v>
+        <v>0.05</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>11.448</v>
+        <v>10.798</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1321.021</v>
+        <v>1419.108</v>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.98</v>
+        <v>0.954</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.065</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>15.035</v>
+        <v>13.443</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1000.586</v>
+        <v>1134.206</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>54.981</v>
+        <v>63.552</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>40.883</v>
+        <v>47.472</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>40.485</v>
+        <v>47.01</v>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>5.69</v>
+        <v>6.607</v>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3114.897</v>
+        <v>3277.13</v>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
@@ -848,7 +848,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3114.897</v>
+        <v>3277.13</v>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>186154.231</v>
+        <v>235149.625</v>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>186154.231</v>
+        <v>235149.625</v>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1322.834</v>
+        <v>1421.055</v>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1322.834</v>
+        <v>1421.055</v>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>97939.541</v>
+        <v>123007.477</v>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
@@ -950,7 +950,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>97939.541</v>
+        <v>123007.477</v>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>15191.953</v>
+        <v>15397.544</v>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
@@ -984,7 +984,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1898.994</v>
+        <v>1924.693</v>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>225815.166</v>
+        <v>246554.573</v>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>28226.896</v>
+        <v>30819.322</v>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>214.845</v>
+        <v>249.328</v>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3.527</v>
+        <v>3.037</v>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>18.623</v>
+        <v>16.111</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>23.149</v>
+        <v>20.148</v>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
@@ -1125,7 +1125,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>3763.586</v>
+        <v>4109.243</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
@@ -1142,7 +1142,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>10941.742</v>
+        <v>11903.028</v>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>30398.053</v>
+        <v>33029.803</v>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
@@ -1176,7 +1176,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>45103.381</v>
+        <v>49042.074</v>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>32646.514</v>
+        <v>41002.492</v>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
@@ -1210,7 +1210,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>77749.895</v>
+        <v>90044.56600000001</v>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>121484.21</v>
+        <v>140694.635</v>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>43734.316</v>
+        <v>50650.069</v>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
@@ -1272,7 +1272,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>16.781</v>
+        <v>15.152</v>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>49.834</v>
+        <v>51.909</v>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
@@ -1306,7 +1306,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>72.32299999999999</v>
+        <v>54.899</v>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
@@ -1323,7 +1323,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>94.41</v>
+        <v>104.954</v>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
@@ -1340,7 +1340,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>197.665</v>
+        <v>220.801</v>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>151.027</v>
+        <v>136.371</v>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>78.992</v>
+        <v>79.178</v>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
@@ -1391,7 +1391,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>111.357</v>
+        <v>80.428</v>
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
@@ -1442,7 +1442,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>303.711</v>
+        <v>351.737</v>
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
@@ -1459,7 +1459,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>852.109</v>
+        <v>825.04</v>
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
@@ -1472,11 +1472,11 @@
       <c r="A64" t="inlineStr"/>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MTOM from model</t>
+          <t>MTOM</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1548.619</v>
+        <v>1569.576</v>
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
@@ -1489,16 +1489,16 @@
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MTOM iterated</t>
+          <t>Battery mass fraction</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1548.619</v>
+        <v>0.224</v>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1506,11 +1506,11 @@
       <c r="A66" t="inlineStr"/>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Battery mass fraction</t>
+          <t>Empty mass fraction</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>0.196</v>
+        <v>0.526</v>
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
@@ -1520,47 +1520,47 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr"/>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Empty mass fraction</t>
-        </is>
-      </c>
-      <c r="C67" t="n">
-        <v>0.55</v>
-      </c>
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>NOISE MODEL</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr">
+      <c r="E67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Thrust coefficient horizontal</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>0.723</v>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>NOISE MODEL</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr"/>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Thrust coefficient horizontal</t>
+          <t>RPM in cruise</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0.529</v>
+        <v>1545.491</v>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>RPM</t>
         </is>
       </c>
     </row>
@@ -1568,16 +1568,16 @@
       <c r="A70" t="inlineStr"/>
       <c r="B70" t="inlineStr">
         <is>
-          <t>RPM in cruise</t>
+          <t>SPL in cruise</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>851.502</v>
+        <v>21.246</v>
       </c>
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
-          <t>RPM</t>
+          <t>dB</t>
         </is>
       </c>
     </row>
@@ -1585,16 +1585,16 @@
       <c r="A71" t="inlineStr"/>
       <c r="B71" t="inlineStr">
         <is>
-          <t>SPL in cruise</t>
+          <t>RPM in climb</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>12.474</v>
+        <v>2346.972</v>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
-          <t>dB</t>
+          <t>RPM</t>
         </is>
       </c>
     </row>
@@ -1602,16 +1602,16 @@
       <c r="A72" t="inlineStr"/>
       <c r="B72" t="inlineStr">
         <is>
-          <t>RPM in climb</t>
+          <t>SPL in climb</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1306.636</v>
+        <v>44.458</v>
       </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
-          <t>RPM</t>
+          <t>dB</t>
         </is>
       </c>
     </row>
@@ -1619,16 +1619,16 @@
       <c r="A73" t="inlineStr"/>
       <c r="B73" t="inlineStr">
         <is>
-          <t>SPL in climb</t>
+          <t>RPM in hover</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>36.218</v>
+        <v>765.178</v>
       </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr">
         <is>
-          <t>dB</t>
+          <t>RPM</t>
         </is>
       </c>
     </row>
@@ -1636,56 +1636,56 @@
       <c r="A74" t="inlineStr"/>
       <c r="B74" t="inlineStr">
         <is>
-          <t>RPM in hover</t>
+          <t>SPL in hover</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>663.8</v>
+        <v>69.982</v>
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
-          <t>RPM</t>
+          <t>dB</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr"/>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>SPL in hover</t>
-        </is>
-      </c>
-      <c r="C75" t="n">
-        <v>67.464</v>
-      </c>
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>BATTERY LIFE MODEL</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>dB</t>
-        </is>
-      </c>
+      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>BATTERY LIFE MODEL</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr"/>
+      <c r="A76" t="inlineStr"/>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>C-rate in hover</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>1.752</v>
+      </c>
       <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>1/h</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr"/>
       <c r="B77" t="inlineStr">
         <is>
-          <t>C-rate in hover</t>
+          <t>C-rate in climb</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1.859</v>
+        <v>1.671</v>
       </c>
       <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
@@ -1698,11 +1698,11 @@
       <c r="A78" t="inlineStr"/>
       <c r="B78" t="inlineStr">
         <is>
-          <t>C-rate in climb</t>
+          <t>C-rate in cruise</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1.532</v>
+        <v>0.874</v>
       </c>
       <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
@@ -1715,11 +1715,11 @@
       <c r="A79" t="inlineStr"/>
       <c r="B79" t="inlineStr">
         <is>
-          <t>C-rate in cruise</t>
+          <t>Time avg. c-rate per trip</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>0.806</v>
+        <v>1.038</v>
       </c>
       <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
@@ -1732,16 +1732,16 @@
       <c r="A80" t="inlineStr"/>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Time avg. c-rate per trip</t>
+          <t>Depth of discharge (DoD)</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>0.962</v>
+        <v>0.349</v>
       </c>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
         <is>
-          <t>1/h</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1749,11 +1749,11 @@
       <c r="A81" t="inlineStr"/>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Depth of discharge (DoD)</t>
+          <t>Battery cycle life</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0.371</v>
+        <v>2592.661</v>
       </c>
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
@@ -1766,11 +1766,11 @@
       <c r="A82" t="inlineStr"/>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Battery cycle life</t>
+          <t>Number of annual battery replacements</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>4983.123</v>
+        <v>1.459</v>
       </c>
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
@@ -1780,42 +1780,42 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr"/>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>Number of annual battery replacements</t>
-        </is>
-      </c>
-      <c r="C83" t="n">
-        <v>0.551</v>
-      </c>
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>OPERATIONS MODEL</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>OPERATIONS MODEL</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr"/>
-      <c r="C84" t="inlineStr"/>
+      <c r="A84" t="inlineStr"/>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Turnaround time</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>12.854</v>
+      </c>
       <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr"/>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Turnaround time</t>
+          <t>Full leg time (flight + turnaround)</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>22.276</v>
+        <v>33.002</v>
       </c>
       <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
@@ -1828,16 +1828,16 @@
       <c r="A86" t="inlineStr"/>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Full leg time (flight + turnaround)</t>
+          <t>Time Efficiency Ratio</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>45.425</v>
+        <v>1.638</v>
       </c>
       <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
-          <t>min</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1845,16 +1845,16 @@
       <c r="A87" t="inlineStr"/>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Time Efficiency Ratio</t>
+          <t>Daily flight cycles</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1.962</v>
+        <v>14.545</v>
       </c>
       <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>flights</t>
         </is>
       </c>
     </row>
@@ -1862,16 +1862,16 @@
       <c r="A88" t="inlineStr"/>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Daily flight cycles</t>
+          <t>Daily flight hours</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>10.567</v>
+        <v>4.884</v>
       </c>
       <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr">
         <is>
-          <t>flights</t>
+          <t>hours</t>
         </is>
       </c>
     </row>
@@ -1879,16 +1879,16 @@
       <c r="A89" t="inlineStr"/>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Daily flight hours</t>
+          <t>Annual flight cycles</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>4.077</v>
+        <v>3781.599</v>
       </c>
       <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
-          <t>hours</t>
+          <t>flights</t>
         </is>
       </c>
     </row>
@@ -1896,56 +1896,56 @@
       <c r="A90" t="inlineStr"/>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Annual flight cycles</t>
+          <t>Annual flight hours</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2747.363</v>
+        <v>1269.877</v>
       </c>
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
-          <t>flights</t>
+          <t>hours</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr"/>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>Annual flight hours</t>
-        </is>
-      </c>
-      <c r="C91" t="n">
-        <v>1059.988</v>
-      </c>
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>GWP MODEL</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr"/>
+      <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr"/>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>hours</t>
-        </is>
-      </c>
+      <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>GWP MODEL</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr"/>
-      <c r="C92" t="inlineStr"/>
+      <c r="A92" t="inlineStr"/>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>GWP of full battery lifecycle</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>17516.482</v>
+      </c>
       <c r="D92" t="inlineStr"/>
-      <c r="E92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>kg CO2e</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr"/>
       <c r="B93" t="inlineStr">
         <is>
-          <t>GWP of full battery lifecycle</t>
+          <t>Ops GWP of battery annually</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>15124.784</v>
+        <v>25549.153</v>
       </c>
       <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr">
@@ -1958,11 +1958,11 @@
       <c r="A94" t="inlineStr"/>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Ops GWP of battery annually</t>
+          <t>Ops GWP of battery per flight</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>8338.800999999999</v>
+        <v>6.756</v>
       </c>
       <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr">
@@ -1975,11 +1975,11 @@
       <c r="A95" t="inlineStr"/>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Ops GWP of battery per flight</t>
+          <t>Ops GWP of energy per flight</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>3.035</v>
+        <v>18.585</v>
       </c>
       <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
@@ -1992,11 +1992,11 @@
       <c r="A96" t="inlineStr"/>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Ops GWP of energy per flight</t>
+          <t>Ops GWP total per flight</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>17.092</v>
+        <v>25.341</v>
       </c>
       <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
@@ -2009,11 +2009,11 @@
       <c r="A97" t="inlineStr"/>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Ops GWP total per flight</t>
+          <t>Ops GWP total per year</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>20.128</v>
+        <v>95830.10400000001</v>
       </c>
       <c r="D97" t="inlineStr"/>
       <c r="E97" t="inlineStr">
@@ -2026,16 +2026,16 @@
       <c r="A98" t="inlineStr"/>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Ops GWP total per year</t>
+          <t>GWP fraction due energy</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>55297.762</v>
+        <v>73.339</v>
       </c>
       <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr">
         <is>
-          <t>kg CO2e</t>
+          <t>%</t>
         </is>
       </c>
     </row>
@@ -2043,11 +2043,11 @@
       <c r="A99" t="inlineStr"/>
       <c r="B99" t="inlineStr">
         <is>
-          <t>GWP fraction due energy</t>
+          <t>GWP fraction due battery</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>84.92</v>
+        <v>26.661</v>
       </c>
       <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr">
@@ -2057,42 +2057,42 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr"/>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>GWP fraction due battery</t>
-        </is>
-      </c>
-      <c r="C100" t="n">
-        <v>15.08</v>
-      </c>
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>ECONOMIC MODEL - COST</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr"/>
+      <c r="C100" t="inlineStr"/>
       <c r="D100" t="inlineStr"/>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
+      <c r="E100" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>ECONOMIC MODEL - COST</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr"/>
-      <c r="C101" t="inlineStr"/>
+      <c r="A101" t="inlineStr"/>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Energy cost per trip</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>4.741</v>
+      </c>
       <c r="D101" t="inlineStr"/>
-      <c r="E101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr"/>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Energy cost per trip</t>
+          <t>Navigation cost per trip</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>4.36</v>
+        <v>17.045</v>
       </c>
       <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr">
@@ -2105,11 +2105,11 @@
       <c r="A103" t="inlineStr"/>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Navigation cost per trip</t>
+          <t>Crew cost per trip</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>16.912</v>
+        <v>12.458</v>
       </c>
       <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr">
@@ -2122,11 +2122,11 @@
       <c r="A104" t="inlineStr"/>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Crew cost per trip</t>
+          <t>Wrap-rated maintenance cost per trip</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>17.148</v>
+        <v>11.082</v>
       </c>
       <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr">
@@ -2139,11 +2139,11 @@
       <c r="A105" t="inlineStr"/>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Wrap-rated maintenance cost per trip</t>
+          <t>Battery unit cost</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>12.732</v>
+        <v>16179.883</v>
       </c>
       <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr">
@@ -2156,11 +2156,11 @@
       <c r="A106" t="inlineStr"/>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Battery unit cost</t>
+          <t>Battery maintenance cost per trip</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>13970.684</v>
+        <v>6.241</v>
       </c>
       <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr">
@@ -2173,11 +2173,11 @@
       <c r="A107" t="inlineStr"/>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Battery maintenance cost per trip</t>
+          <t>Total maintenance cost per trip</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>2.804</v>
+        <v>17.322</v>
       </c>
       <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr">
@@ -2190,11 +2190,11 @@
       <c r="A108" t="inlineStr"/>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Total maintenance cost per trip</t>
+          <t>Cash operating cost per trip</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>15.536</v>
+        <v>51.566</v>
       </c>
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr">
@@ -2207,11 +2207,11 @@
       <c r="A109" t="inlineStr"/>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Cash operating cost per trip</t>
+          <t>Cost of ownership per trip</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>53.956</v>
+        <v>28.041</v>
       </c>
       <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr">
@@ -2224,11 +2224,11 @@
       <c r="A110" t="inlineStr"/>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Cost of ownership per trip</t>
+          <t>Direct operating cost per trip</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>38.702</v>
+        <v>79.607</v>
       </c>
       <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr">
@@ -2241,11 +2241,11 @@
       <c r="A111" t="inlineStr"/>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Direct operating cost per trip</t>
+          <t>Indirect operating cost per trip</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>92.658</v>
+        <v>17.5</v>
       </c>
       <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr">
@@ -2258,11 +2258,11 @@
       <c r="A112" t="inlineStr"/>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Indirect operating cost per trip</t>
+          <t>Total operating cost per trip</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>20.369</v>
+        <v>97.107</v>
       </c>
       <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr">
@@ -2275,16 +2275,16 @@
       <c r="A113" t="inlineStr"/>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Total operating cost per trip</t>
+          <t>TOC per available seat per km</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>113.027</v>
+        <v>0.347</v>
       </c>
       <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr">
         <is>
-          <t>€</t>
+          <t>€/km</t>
         </is>
       </c>
     </row>
@@ -2292,56 +2292,56 @@
       <c r="A114" t="inlineStr"/>
       <c r="B114" t="inlineStr">
         <is>
-          <t>TOC per available seat per km</t>
+          <t>TOC per available seat per min</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>0.404</v>
+        <v>1.205</v>
       </c>
       <c r="D114" t="inlineStr"/>
       <c r="E114" t="inlineStr">
         <is>
-          <t>€/km</t>
+          <t>€/min</t>
         </is>
       </c>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr"/>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>TOC per available seat per min</t>
-        </is>
-      </c>
-      <c r="C115" t="n">
-        <v>1.221</v>
-      </c>
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>ECONOMIC MODEL - REVENUE</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr"/>
+      <c r="C115" t="inlineStr"/>
       <c r="D115" t="inlineStr"/>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>€/min</t>
-        </is>
-      </c>
+      <c r="E115" t="inlineStr"/>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>ECONOMIC MODEL - REVENUE</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr"/>
-      <c r="C116" t="inlineStr"/>
+      <c r="A116" t="inlineStr"/>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Ticket price per pax per trip</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>138.6</v>
+      </c>
       <c r="D116" t="inlineStr"/>
-      <c r="E116" t="inlineStr"/>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr"/>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Ticket price per pax per trip</t>
+          <t>Revenue per trip</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>138.6</v>
+        <v>376.992</v>
       </c>
       <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr">
@@ -2351,62 +2351,45 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr"/>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>Revenue per trip</t>
-        </is>
-      </c>
-      <c r="C118" t="n">
-        <v>376.992</v>
-      </c>
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>ECONOMIC MODEL - PROFIT</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr"/>
+      <c r="C118" t="inlineStr"/>
       <c r="D118" t="inlineStr"/>
-      <c r="E118" t="inlineStr">
+      <c r="E118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr"/>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Total profit per trip</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>279.885</v>
+      </c>
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>ECONOMIC MODEL - PROFIT</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr"/>
-      <c r="C119" t="inlineStr"/>
-      <c r="D119" t="inlineStr"/>
-      <c r="E119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr"/>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Total profit per trip</t>
+          <t>Total profit per year</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>263.965</v>
+        <v>1058413.296</v>
       </c>
       <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr"/>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>Total profit per year</t>
-        </is>
-      </c>
-      <c r="C121" t="n">
-        <v>725208.77</v>
-      </c>
-      <c r="D121" t="inlineStr"/>
-      <c r="E121" t="inlineStr">
         <is>
           <t>€</t>
         </is>
@@ -2485,13 +2468,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7.745</v>
+        <v>7.717</v>
       </c>
       <c r="C2" t="n">
         <v>64.235</v>
       </c>
       <c r="D2" t="n">
-        <v>8.593</v>
+        <v>8.507</v>
       </c>
       <c r="E2" t="n">
         <v>1.183</v>
@@ -2519,13 +2502,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7.564</v>
+        <v>7.535</v>
       </c>
       <c r="C3" t="n">
         <v>64.235</v>
       </c>
       <c r="D3" t="n">
-        <v>8.593</v>
+        <v>8.507</v>
       </c>
       <c r="E3" t="n">
         <v>2.366</v>
@@ -2553,13 +2536,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7.479</v>
+        <v>7.448</v>
       </c>
       <c r="C4" t="n">
         <v>50.909</v>
       </c>
       <c r="D4" t="n">
-        <v>9.048999999999999</v>
+        <v>8.958</v>
       </c>
       <c r="E4" t="n">
         <v>0.588</v>
@@ -2587,13 +2570,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7.47</v>
+        <v>7.442</v>
       </c>
       <c r="C5" t="n">
         <v>64.235</v>
       </c>
       <c r="D5" t="n">
-        <v>8.593</v>
+        <v>8.507</v>
       </c>
       <c r="E5" t="n">
         <v>2.821</v>
@@ -2621,13 +2604,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7.068</v>
+        <v>7.045</v>
       </c>
       <c r="C6" t="n">
         <v>105</v>
       </c>
       <c r="D6" t="n">
-        <v>7.197</v>
+        <v>7.127</v>
       </c>
       <c r="E6" t="n">
         <v>1.456</v>
@@ -2651,69 +2634,69 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Electric Vehicle (26%)</t>
+          <t>Bicycle</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7.004</v>
+        <v>6.999</v>
       </c>
       <c r="C7" t="n">
-        <v>64.235</v>
+        <v>285.957</v>
       </c>
       <c r="D7" t="n">
-        <v>8.593</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>4.55</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>7.762</v>
+        <v>10</v>
       </c>
       <c r="G7" t="n">
-        <v>12089.35</v>
+        <v>-9955.456</v>
       </c>
       <c r="H7" t="n">
-        <v>7.061</v>
+        <v>10</v>
       </c>
       <c r="I7" t="n">
-        <v>7.371</v>
+        <v>-43.994</v>
       </c>
       <c r="J7" t="n">
-        <v>4.659</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bicycle</t>
+          <t>Electric Vehicle (26%)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6.999</v>
+        <v>6.975</v>
       </c>
       <c r="C8" t="n">
-        <v>285.957</v>
+        <v>64.235</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>8.507</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>4.55</v>
       </c>
       <c r="F8" t="n">
-        <v>10</v>
+        <v>7.762</v>
       </c>
       <c r="G8" t="n">
-        <v>-9955.456</v>
+        <v>12089.35</v>
       </c>
       <c r="H8" t="n">
-        <v>10</v>
+        <v>7.061</v>
       </c>
       <c r="I8" t="n">
-        <v>-43.994</v>
+        <v>7.371</v>
       </c>
       <c r="J8" t="n">
-        <v>10</v>
+        <v>4.659</v>
       </c>
     </row>
     <row r="9">
@@ -2723,13 +2706,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6.822</v>
+        <v>6.792</v>
       </c>
       <c r="C9" t="n">
         <v>50.909</v>
       </c>
       <c r="D9" t="n">
-        <v>9.048999999999999</v>
+        <v>8.958</v>
       </c>
       <c r="E9" t="n">
         <v>1.008</v>
@@ -2757,13 +2740,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6.732</v>
+        <v>6.709</v>
       </c>
       <c r="C10" t="n">
         <v>105</v>
       </c>
       <c r="D10" t="n">
-        <v>7.197</v>
+        <v>7.127</v>
       </c>
       <c r="E10" t="n">
         <v>2.464</v>
@@ -2791,13 +2774,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6.705</v>
+        <v>6.676</v>
       </c>
       <c r="C11" t="n">
         <v>64.235</v>
       </c>
       <c r="D11" t="n">
-        <v>8.593</v>
+        <v>8.507</v>
       </c>
       <c r="E11" t="n">
         <v>5.915</v>
@@ -2825,13 +2808,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.327</v>
+        <v>6.298</v>
       </c>
       <c r="C12" t="n">
         <v>64.235</v>
       </c>
       <c r="D12" t="n">
-        <v>8.593</v>
+        <v>8.507</v>
       </c>
       <c r="E12" t="n">
         <v>9.009</v>
@@ -2859,13 +2842,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5.932</v>
+        <v>5.903</v>
       </c>
       <c r="C13" t="n">
         <v>64.235</v>
       </c>
       <c r="D13" t="n">
-        <v>8.593</v>
+        <v>8.507</v>
       </c>
       <c r="E13" t="n">
         <v>10.92</v>
@@ -2893,13 +2876,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5.834</v>
+        <v>5.806</v>
       </c>
       <c r="C14" t="n">
         <v>64.235</v>
       </c>
       <c r="D14" t="n">
-        <v>8.593</v>
+        <v>8.507</v>
       </c>
       <c r="E14" t="n">
         <v>11.648</v>
@@ -2927,31 +2910,31 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5.821</v>
+        <v>5.71</v>
       </c>
       <c r="C15" t="n">
-        <v>23.149</v>
+        <v>20.148</v>
       </c>
       <c r="D15" t="n">
         <v>10</v>
       </c>
       <c r="E15" t="n">
-        <v>7.4</v>
+        <v>9.317</v>
       </c>
       <c r="F15" t="n">
-        <v>6.361</v>
+        <v>5.418</v>
       </c>
       <c r="G15" t="n">
-        <v>16582.125</v>
+        <v>18030.174</v>
       </c>
       <c r="H15" t="n">
-        <v>6.462</v>
+        <v>6.269</v>
       </c>
       <c r="I15" t="n">
-        <v>41.554</v>
+        <v>35.701</v>
       </c>
       <c r="J15" t="n">
-        <v>1.104</v>
+        <v>1.713</v>
       </c>
     </row>
     <row r="16">
@@ -2961,13 +2944,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5.295</v>
+        <v>5.266</v>
       </c>
       <c r="C16" t="n">
         <v>64.235</v>
       </c>
       <c r="D16" t="n">
-        <v>8.593</v>
+        <v>8.507</v>
       </c>
       <c r="E16" t="n">
         <v>14.287</v>
@@ -2995,13 +2978,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3.131</v>
+        <v>3.118</v>
       </c>
       <c r="C17" t="n">
         <v>179.595</v>
       </c>
       <c r="D17" t="n">
-        <v>4.642</v>
+        <v>4.601</v>
       </c>
       <c r="E17" t="n">
         <v>14.553</v>
@@ -3029,13 +3012,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2.214</v>
+        <v>2.2</v>
       </c>
       <c r="C18" t="n">
         <v>179.595</v>
       </c>
       <c r="D18" t="n">
-        <v>4.642</v>
+        <v>4.601</v>
       </c>
       <c r="E18" t="n">
         <v>18.302</v>

</xml_diff>